<commit_message>
revisi logic parser tgl muat , revisi tgl 09/03/2025
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="172">
   <si>
     <t>DATE</t>
   </si>
@@ -37,82 +37,644 @@
     <t>PLATE</t>
   </si>
   <si>
+    <t>TIME</t>
+  </si>
+  <si>
     <t>Original_Text</t>
   </si>
   <si>
     <t>PHONE</t>
   </si>
   <si>
-    <t>3 maret 2026</t>
-  </si>
-  <si>
-    <t>18 maret 2026</t>
+    <t>06 febuary 2026</t>
+  </si>
+  <si>
+    <t>06 feb 2026</t>
+  </si>
+  <si>
+    <t>06 febuari 2026</t>
+  </si>
+  <si>
+    <t>07 febuari 2026</t>
+  </si>
+  <si>
+    <t>08 februari 2025</t>
+  </si>
+  <si>
+    <t>09 feb</t>
+  </si>
+  <si>
+    <t>9 februari 2026</t>
+  </si>
+  <si>
+    <t>10 / 02 / 2026</t>
+  </si>
+  <si>
+    <t>11 februari 2026</t>
+  </si>
+  <si>
+    <t>09 : 00 11 februari 2026</t>
+  </si>
+  <si>
+    <t>12 februari 2026</t>
+  </si>
+  <si>
+    <t>12 / 02 / 2026</t>
+  </si>
+  <si>
+    <t>12 feb 26</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>twb</t>
+  </si>
+  <si>
     <t>wb</t>
   </si>
   <si>
-    <t>cbm</t>
+    <t>cddl</t>
+  </si>
+  <si>
+    <t>jne</t>
   </si>
   <si>
     <t>argopantes</t>
   </si>
   <si>
+    <t>cikokol</t>
+  </si>
+  <si>
+    <t>megahub</t>
+  </si>
+  <si>
+    <t>cikarang</t>
+  </si>
+  <si>
+    <t>subcgk</t>
+  </si>
+  <si>
     <t>cgk sub</t>
   </si>
   <si>
-    <t>sub cgk</t>
+    <t>cgk tentatif</t>
+  </si>
+  <si>
+    <t>cgk mes</t>
+  </si>
+  <si>
+    <t>cgk pku</t>
+  </si>
+  <si>
+    <t>srg sub</t>
+  </si>
+  <si>
+    <t>jne srg</t>
+  </si>
+  <si>
+    <t>srgcgk</t>
+  </si>
+  <si>
+    <t>cgk dps</t>
+  </si>
+  <si>
+    <t>cgk</t>
+  </si>
+  <si>
+    <t>ckrsubsux</t>
+  </si>
+  <si>
+    <t>cgkjbr</t>
+  </si>
+  <si>
+    <t>akbar</t>
+  </si>
+  <si>
+    <t>wahyudi</t>
   </si>
   <si>
     <t>sofyan</t>
   </si>
   <si>
+    <t>chandra</t>
+  </si>
+  <si>
+    <t>sentot</t>
+  </si>
+  <si>
+    <t>purwanto</t>
+  </si>
+  <si>
+    <t>didik</t>
+  </si>
+  <si>
+    <t>haryono</t>
+  </si>
+  <si>
+    <t>hermanto</t>
+  </si>
+  <si>
+    <t>wijaya</t>
+  </si>
+  <si>
+    <t>darmawan</t>
+  </si>
+  <si>
+    <t>arif r</t>
+  </si>
+  <si>
     <t>yuda</t>
   </si>
   <si>
-    <t>b 9679wt</t>
+    <t>aldi</t>
+  </si>
+  <si>
+    <t>supriadi</t>
+  </si>
+  <si>
+    <t>syafrizal</t>
+  </si>
+  <si>
+    <t>nizar</t>
+  </si>
+  <si>
+    <t>samosir</t>
+  </si>
+  <si>
+    <t>joni</t>
+  </si>
+  <si>
+    <t>nasip k</t>
+  </si>
+  <si>
+    <t>ageng</t>
+  </si>
+  <si>
+    <t>ilham wahyudi</t>
+  </si>
+  <si>
+    <t>sri mardono</t>
+  </si>
+  <si>
+    <t>n 9549 ua</t>
+  </si>
+  <si>
+    <t>b 9679 wt</t>
+  </si>
+  <si>
+    <t>l 8601 uh</t>
+  </si>
+  <si>
+    <t>b 9231 ceu</t>
+  </si>
+  <si>
+    <t>b 9891 beu</t>
+  </si>
+  <si>
+    <t>b 9687 jm</t>
+  </si>
+  <si>
+    <t>b 8745 amr</t>
+  </si>
+  <si>
+    <t>s 8635 nj</t>
+  </si>
+  <si>
+    <t>h 9948 ra</t>
+  </si>
+  <si>
+    <t>ba 8829 bu</t>
+  </si>
+  <si>
+    <t>b 9787 xx</t>
   </si>
   <si>
     <t>w 8973 uq</t>
   </si>
   <si>
-    <t>REQUEST  ORDER  ONCALL  3 MARET 2026
+    <t>bm 8350 au</t>
+  </si>
+  <si>
+    <t>b 9586 txv</t>
+  </si>
+  <si>
+    <t>bm 8479 au</t>
+  </si>
+  <si>
+    <t>b 9172 scp</t>
+  </si>
+  <si>
+    <t>b 9727 uex</t>
+  </si>
+  <si>
+    <t>b 9169 uex</t>
+  </si>
+  <si>
+    <t>bh 8165 qi</t>
+  </si>
+  <si>
+    <t>b9654yu</t>
+  </si>
+  <si>
+    <t>f 9647 fh</t>
+  </si>
+  <si>
+    <t>bk 8678 ve</t>
+  </si>
+  <si>
+    <t>segera</t>
+  </si>
+  <si>
+    <t>07 : 00</t>
+  </si>
+  <si>
+    <t>22 : 00</t>
+  </si>
+  <si>
+    <t>02 : 00</t>
+  </si>
+  <si>
+    <t>03 : 00</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 06 febuary 2026
+2 unit twb 50 CBM
+Lokasi : JNE SUB</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 06 febuary 2026
+Rute/tujuan : SUB-CGK
+driver  : WAHYUDI
+Nopol  : N 9549 UA
+No hp  :085784422398</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 06 febuary 2026
+Rute/tujuan : SUB-CGK
+driver  : SOFYAN
+Nopol  : B 9679 WT
+No hp  : 082231837381</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+06 FEB 2026
 6 UNIT WB/50 CBM
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading : 23:00 3 MARET 2026
-Rute/tujuan : CGK - SUB 
-driver  : Rosyit
-Nopol  : B 9562 TEU
-No hp  : 082313572678
-Driver : sofyan
-Nopol : B 9679WT
-No Hp : 082231837381</t>
-  </si>
-  <si>
-    <t>REQUEST  ORDER  ONCALL  18 MARET 2026
-1 UNIT WB/50 CBM
+    <t>REQUEST ORDER KHUSUS 07-02-2026</t>
+  </si>
+  <si>
+    <t>Waktu loading : 07:00
+Rute/tujuan : CGK - SUB
+driver  : Chandra
+Nopol  : L 8601 UH
+No hp  : +62 852-3168-1470</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+06 FEB 2026
+10 UNIT CDDL/24 CBM
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading : 23:00 18 MARET 2026
-Rute/tujuan : SUB - CGK
-driver  : Yuda
-Nopol  : W 8973 UQ
-No hp  : 089507296985</t>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CGK - JATIM TENTATIF</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCAL
+06 FEBUARI 2026
+RAFAY
+3 unit TWB 50 Cbm
+Lokasi : ARGOPANTES
+Rute/ tuj : CGK - MES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+DRIVER 1 : SENTOT
+NOPOL    : B 9231 CEU
+NOHP      :+62 812-8714-7789</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCAL
+06 FEBUARI 2026
+5 unit TWB 50 Cbm
+Lokasi : ARGOPANTES
+Rute/ tuj : CGK - SUB</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+RAFAY
+DRIVER 1 : PURWANTO
+NOPOL    : B 9891 BEU
+NOHP      :083142142113</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+DRIVER : DIDIK
+NOPOL    : B 9687 JM
+NOHP      :085385220743</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCAL
+06 FEBUARI 2026
+Lokasi : ARGOPANTES
+Rute/ tuj : CGK - PKU</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+DRIVER 1 : Haryono
+NOPOL    : B 8745 AMR
+NO HP      : 083166684195</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+DRIVER : HERMANTO
+NOPOL : S 8635 NJ
+NOHP :085194592825</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCAL
+07 FEBUARI 2026
+RAFAY
+1 unit CDDL 24 Cbm
+Lokasi : SEMARANG
+Rute/ tuj : SRG - SUB</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+DRIVER 1 :Agung
+DRIVER 2 :Wijaya
+NOPOL    :H 9948 RA
+NOHP      :0882016641381</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 08 FEBRUARI 2025:
+3 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 08 FEBRUARI 2025
+Rute/tujuan : CGK - MES
+driver  : DARMAWAN
+Nopol  : BA 8829 BU
+No hp  :082363564665</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Order Oncall Tgl 09 Feb
+1 UNIT CDDL 24 CBM
+Lokasi  : JNE SRG</t>
+  </si>
+  <si>
+    <t>Waktu loading : 22:00
+Rute/tujuan : SRG-CGK
+Driver : Arif R
+Nopol :B 9787 XX
+No hp :089690885555</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER  ONCALL 9 FEBRUARI 2026:
+2 unit TWB 50 Cbm
+Lokasi : cikokol</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER KHUSUS 10/02/2026</t>
+  </si>
+  <si>
+    <t>Waktu loading : 02:00
+Rute/tujuan : CGK - SUB
+NAMA : WAHYUDI
+NOPOL: N 9549 UA
+NO HP :085784422398</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00
+NAMA : YUDA
+NOPOL: W 8973 UQ
+NO HP :089507296985</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER  ONCALL 9 FEBRUARI 2026:
+2 unit  TWB 50 Cbm
+Lokasi : Cikokol</t>
+  </si>
+  <si>
+    <t>Waktu loading : 02:00
+Rute/tujuan : CGK - PKU
+NAMA : ALDI
+NOPOL: BM 8350 AU
+NO HP :0831-6761-0479</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00
+NAMA :
+NOPOL:
+NO HP :</t>
+  </si>
+  <si>
+    <t>Waktu loading : 02:00
+Rute/tujuan : SRG-CGK
+Driver : Supriadi
+Nopol : B 9586 TXV
+No hp :081350529712</t>
+  </si>
+  <si>
+    <t>Waktu loading : 02:00
+Rute/tujuan : CGK - PKU</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00
+NAMA : SYAFRIZAL
+NOPOL: BM 8479 AU
+NO HP :082170733190</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER  ONCALL 9 FEBRUARI 2026:
+RAFAY
+2 unit  TWB 50 Cbm
+Lokasi : Cikokol
+Rute/tujuan : CGK - PKU</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 9 FEBRUARI 2026
+NAMA : SYAFRIZAL
+NOPOL: BM 8479 AU
+NO HP :082170733190</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 11 FEBRUARI 2026:
+1 unit Cddl 24 Cbm
+Lokasi : Megahub</t>
+  </si>
+  <si>
+    <t>Waktu loading : 00:00 11 FEBRUARI 2026
+Rute/tujuan : CGK - DPS
+driver  :Nizar
+Nopol  :B 9172 SCP
+No hp  :081313444015</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 11 FEBRUARI 2026:
+3 unit tronton 50 Cbm
+Lokasi : cikokol</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 11 FEBRUARI 2026
+Rute/tujuan : CGK - MES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 09:00 11 FEBRUARI 2026
+Driver : SAMOSIR
+Nopol : B 9727 UEX
+Hp :+62 822-7429-6236</t>
+  </si>
+  <si>
+    <t>Waktu loading : 12:00 11 FEBRUARI 2026
+Driver : JONI
+Nopol : B 9169 UEX
+Hp :+62 822-7638-5077</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER TAMBAHAN ONCALL  12 FEBRUARI 2026:
+1 unit TRONTON 50 Cbm
+Lokasi : cikokol</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER KHUSUS 12/02/2026</t>
+  </si>
+  <si>
+    <t>Waktu loading : 02:00
+Rute/tujuan : CGK - PKU
+Nama 	: NASIP K
+Nopol		: BH 8165 QI
+No Tlp		:‪+6281272463920</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 12 Feb 26
+1 Unit  TWB 50 Cbm
+Lokasi : Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CKR-SUB-SUX 
+Driver   : AGENG
+Nopol  : B9654YU
+No Hp  : +62 857-0738-0584</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 12 Feb 26
+1 Unit  Cddl / 24 Cbm
+Lokasi : Cikokol + Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00
+Rute/tujuan : CGK-JBR
+No pol.   : F 9647 FH
+Driver. 1 :  Jatmiyanta
+No hp :  : 082118558105
+Driver 2  : Ilham Wahyudi
+No hp.    : 089519041791</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 12 FEBRUARI 2026:
+RAFAY
+3 unit tronton 50 Cbm
+Lokasi : cikokol</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 12 FEBRUARI 2026
+Rute/tujuan : CGK - MES
+driver  : SRI MARDONO
+Nopol  : BK 8678 VE
+No hp  :085218843366</t>
+  </si>
+  <si>
+    <t>085784422398</t>
   </si>
   <si>
     <t>082231837381</t>
   </si>
   <si>
+    <t>07022026</t>
+  </si>
+  <si>
+    <t>0 85231681470</t>
+  </si>
+  <si>
+    <t>0 81287147789</t>
+  </si>
+  <si>
+    <t>083142142113</t>
+  </si>
+  <si>
+    <t>085385220743</t>
+  </si>
+  <si>
+    <t>083166684195</t>
+  </si>
+  <si>
+    <t>085194592825</t>
+  </si>
+  <si>
+    <t>0882016641381</t>
+  </si>
+  <si>
+    <t>082363564665</t>
+  </si>
+  <si>
+    <t>089690885555</t>
+  </si>
+  <si>
     <t>089507296985</t>
+  </si>
+  <si>
+    <t>083167610479</t>
+  </si>
+  <si>
+    <t>081350529712</t>
+  </si>
+  <si>
+    <t>082170733190</t>
+  </si>
+  <si>
+    <t>081313444015</t>
+  </si>
+  <si>
+    <t>0 82274296236</t>
+  </si>
+  <si>
+    <t>0 82276385077</t>
+  </si>
+  <si>
+    <t>081272463920</t>
+  </si>
+  <si>
+    <t>0 85707380584</t>
+  </si>
+  <si>
+    <t>089519041791</t>
+  </si>
+  <si>
+    <t>085218843366</t>
   </si>
 </sst>
 </file>
@@ -470,10 +1032,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,79 +1063,993 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>101</v>
+      </c>
+      <c r="J3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" t="s">
+        <v>95</v>
+      </c>
+      <c r="I5" t="s">
+        <v>102</v>
+      </c>
+      <c r="J5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="I7" t="s">
+        <v>104</v>
+      </c>
+      <c r="J7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="E10" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" t="s">
+        <v>95</v>
+      </c>
+      <c r="I10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="F12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" t="s">
+        <v>95</v>
+      </c>
+      <c r="I12" t="s">
+        <v>109</v>
+      </c>
+      <c r="J12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="F14" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" t="s">
+        <v>77</v>
+      </c>
+      <c r="H14" t="s">
+        <v>95</v>
+      </c>
+      <c r="I14" t="s">
+        <v>111</v>
+      </c>
+      <c r="J14" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="F16" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" t="s">
+        <v>95</v>
+      </c>
+      <c r="I16" t="s">
+        <v>112</v>
+      </c>
+      <c r="J16" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I17" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" t="s">
+        <v>95</v>
+      </c>
+      <c r="I18" t="s">
+        <v>114</v>
+      </c>
+      <c r="J18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" t="s">
+        <v>39</v>
+      </c>
+      <c r="F19" t="s">
+        <v>50</v>
+      </c>
+      <c r="I19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="F20" t="s">
+        <v>58</v>
+      </c>
+      <c r="G20" t="s">
+        <v>80</v>
+      </c>
+      <c r="H20" t="s">
+        <v>95</v>
+      </c>
+      <c r="I20" t="s">
+        <v>115</v>
+      </c>
+      <c r="J20" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" t="s">
+        <v>43</v>
+      </c>
+      <c r="I21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="F22" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" t="s">
+        <v>81</v>
+      </c>
+      <c r="H22" t="s">
+        <v>95</v>
+      </c>
+      <c r="I22" t="s">
+        <v>117</v>
+      </c>
+      <c r="J22" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I23" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>82</v>
+      </c>
+      <c r="H24" t="s">
+        <v>95</v>
+      </c>
+      <c r="I24" t="s">
+        <v>119</v>
+      </c>
+      <c r="J24" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" t="s">
+        <v>44</v>
+      </c>
+      <c r="I25" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="E26" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" t="s">
+        <v>61</v>
+      </c>
+      <c r="G26" t="s">
+        <v>83</v>
+      </c>
+      <c r="H26" t="s">
+        <v>97</v>
+      </c>
+      <c r="I26" t="s">
+        <v>121</v>
+      </c>
+      <c r="J26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" t="s">
+        <v>35</v>
+      </c>
+      <c r="I27" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" t="s">
         <v>17</v>
       </c>
-      <c r="F5" t="s">
+      <c r="I28" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="E29" t="s">
+        <v>39</v>
+      </c>
+      <c r="F29" t="s">
+        <v>51</v>
+      </c>
+      <c r="G29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" t="s">
+        <v>98</v>
+      </c>
+      <c r="I29" t="s">
+        <v>124</v>
+      </c>
+      <c r="J29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="F31" t="s">
+        <v>62</v>
+      </c>
+      <c r="G31" t="s">
+        <v>84</v>
+      </c>
+      <c r="H31" t="s">
+        <v>99</v>
+      </c>
+      <c r="I31" t="s">
+        <v>125</v>
+      </c>
+      <c r="J31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C32" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" t="s">
+        <v>35</v>
+      </c>
+      <c r="I32" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="E34" t="s">
+        <v>42</v>
+      </c>
+      <c r="F34" t="s">
+        <v>63</v>
+      </c>
+      <c r="G34" t="s">
+        <v>85</v>
+      </c>
+      <c r="H34" t="s">
+        <v>98</v>
+      </c>
+      <c r="I34" t="s">
+        <v>127</v>
+      </c>
+      <c r="J34" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="H36" t="s">
+        <v>99</v>
+      </c>
+      <c r="I36" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
+      <c r="A37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37" t="s">
+        <v>44</v>
+      </c>
+      <c r="I37" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
+      <c r="E38" t="s">
+        <v>45</v>
+      </c>
+      <c r="F38" t="s">
+        <v>64</v>
+      </c>
+      <c r="G38" t="s">
+        <v>86</v>
+      </c>
+      <c r="H38" t="s">
+        <v>98</v>
+      </c>
+      <c r="I38" t="s">
+        <v>129</v>
+      </c>
+      <c r="J38" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
+      <c r="A39" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" t="s">
+        <v>30</v>
+      </c>
+      <c r="D39" t="s">
+        <v>35</v>
+      </c>
+      <c r="I39" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10">
+      <c r="A40" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
+      <c r="E41" t="s">
+        <v>42</v>
+      </c>
+      <c r="H41" t="s">
+        <v>98</v>
+      </c>
+      <c r="I41" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="I42" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
+      <c r="F43" t="s">
+        <v>65</v>
+      </c>
+      <c r="G43" t="s">
+        <v>87</v>
+      </c>
+      <c r="H43" t="s">
+        <v>99</v>
+      </c>
+      <c r="I43" t="s">
+        <v>131</v>
+      </c>
+      <c r="J43" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10">
+      <c r="A44" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" t="s">
+        <v>30</v>
+      </c>
+      <c r="D44" t="s">
+        <v>35</v>
+      </c>
+      <c r="E44" t="s">
+        <v>42</v>
+      </c>
+      <c r="I44" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10">
+      <c r="A45" t="s">
+        <v>16</v>
+      </c>
+      <c r="F45" t="s">
+        <v>65</v>
+      </c>
+      <c r="G45" t="s">
+        <v>87</v>
+      </c>
+      <c r="H45" t="s">
+        <v>95</v>
+      </c>
+      <c r="I45" t="s">
+        <v>133</v>
+      </c>
+      <c r="J45" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10">
+      <c r="A46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C46" t="s">
+        <v>32</v>
+      </c>
+      <c r="D46" t="s">
+        <v>36</v>
+      </c>
+      <c r="I46" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" t="s">
+        <v>18</v>
+      </c>
+      <c r="E47" t="s">
+        <v>46</v>
+      </c>
+      <c r="F47" t="s">
+        <v>66</v>
+      </c>
+      <c r="G47" t="s">
+        <v>88</v>
+      </c>
+      <c r="I47" t="s">
+        <v>135</v>
+      </c>
+      <c r="J47" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" t="s">
+        <v>18</v>
+      </c>
+      <c r="B48" t="s">
+        <v>29</v>
+      </c>
+      <c r="D48" t="s">
+        <v>35</v>
+      </c>
+      <c r="I48" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" t="s">
+        <v>18</v>
+      </c>
+      <c r="E49" t="s">
+        <v>47</v>
+      </c>
+      <c r="H49" t="s">
+        <v>95</v>
+      </c>
+      <c r="I49" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" t="s">
         <v>19</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F50" t="s">
+        <v>67</v>
+      </c>
+      <c r="G50" t="s">
+        <v>89</v>
+      </c>
+      <c r="I50" t="s">
+        <v>138</v>
+      </c>
+      <c r="J50" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" t="s">
+        <v>18</v>
+      </c>
+      <c r="F51" t="s">
+        <v>68</v>
+      </c>
+      <c r="G51" t="s">
+        <v>90</v>
+      </c>
+      <c r="I51" t="s">
+        <v>139</v>
+      </c>
+      <c r="J51" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
+      <c r="A52" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" t="s">
+        <v>29</v>
+      </c>
+      <c r="D52" t="s">
+        <v>35</v>
+      </c>
+      <c r="I52" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
+      <c r="A53" t="s">
         <v>21</v>
       </c>
-      <c r="H5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I5" t="s">
-        <v>27</v>
+      <c r="I53" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
+      <c r="E54" t="s">
+        <v>42</v>
+      </c>
+      <c r="F54" t="s">
+        <v>69</v>
+      </c>
+      <c r="G54" t="s">
+        <v>91</v>
+      </c>
+      <c r="H54" t="s">
+        <v>98</v>
+      </c>
+      <c r="I54" t="s">
+        <v>142</v>
+      </c>
+      <c r="J54" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
+      <c r="A55" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55" t="s">
+        <v>30</v>
+      </c>
+      <c r="D55" t="s">
+        <v>37</v>
+      </c>
+      <c r="F55" t="s">
+        <v>50</v>
+      </c>
+      <c r="I55" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
+      <c r="E56" t="s">
+        <v>48</v>
+      </c>
+      <c r="F56" t="s">
+        <v>70</v>
+      </c>
+      <c r="G56" t="s">
+        <v>92</v>
+      </c>
+      <c r="H56" t="s">
+        <v>95</v>
+      </c>
+      <c r="I56" t="s">
+        <v>144</v>
+      </c>
+      <c r="J56" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
+      <c r="A57" t="s">
+        <v>22</v>
+      </c>
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" t="s">
+        <v>32</v>
+      </c>
+      <c r="E57" t="s">
+        <v>37</v>
+      </c>
+      <c r="F57" t="s">
+        <v>50</v>
+      </c>
+      <c r="I57" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
+      <c r="E58" t="s">
+        <v>49</v>
+      </c>
+      <c r="F58" t="s">
+        <v>71</v>
+      </c>
+      <c r="G58" t="s">
+        <v>93</v>
+      </c>
+      <c r="H58" t="s">
+        <v>99</v>
+      </c>
+      <c r="I58" t="s">
+        <v>146</v>
+      </c>
+      <c r="J58" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" t="s">
+        <v>26</v>
+      </c>
+      <c r="D59" t="s">
+        <v>35</v>
+      </c>
+      <c r="I59" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" t="s">
+        <v>20</v>
+      </c>
+      <c r="E60" t="s">
+        <v>41</v>
+      </c>
+      <c r="F60" t="s">
+        <v>72</v>
+      </c>
+      <c r="G60" t="s">
+        <v>94</v>
+      </c>
+      <c r="H60" t="s">
+        <v>95</v>
+      </c>
+      <c r="I60" t="s">
+        <v>148</v>
+      </c>
+      <c r="J60" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
revisi logic parser tujuan, pickup, tgl muat
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="172">
   <si>
     <t>DATE</t>
   </si>
@@ -457,17 +457,14 @@
 Lokasi : cikokol</t>
   </si>
   <si>
-    <t>REQUEST ORDER KHUSUS 10/02/2026</t>
-  </si>
-  <si>
-    <t>Waktu loading : 02:00
+    <t>Waktu loading : 02:00 9 FEBRUARI 2026
 Rute/tujuan : CGK - SUB
 NAMA : WAHYUDI
 NOPOL: N 9549 UA
 NO HP :085784422398</t>
   </si>
   <si>
-    <t>Waktu loading : 03:00
+    <t>Waktu loading : 03:00 9 FEBRUARI 2026
 NAMA : YUDA
 NOPOL: W 8973 UQ
 NO HP :089507296985</t>
@@ -476,6 +473,9 @@
     <t>[WA_TS] Akbar Rafay: REQUEST ORDER  ONCALL 9 FEBRUARI 2026:
 2 unit  TWB 50 Cbm
 Lokasi : Cikokol</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER KHUSUS 10/02/2026</t>
   </si>
   <si>
     <t>Waktu loading : 02:00
@@ -1032,7 +1032,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1544,72 +1544,84 @@
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="E28" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" t="s">
+        <v>73</v>
       </c>
       <c r="I28" t="s">
         <v>123</v>
       </c>
+      <c r="J28" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="29" spans="1:10">
-      <c r="E29" t="s">
-        <v>39</v>
+      <c r="A29" t="s">
+        <v>16</v>
       </c>
       <c r="F29" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="G29" t="s">
-        <v>73</v>
-      </c>
-      <c r="H29" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="I29" t="s">
         <v>124</v>
       </c>
       <c r="J29" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" t="s">
+        <v>35</v>
+      </c>
+      <c r="I30" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" t="s">
         <v>17</v>
       </c>
-      <c r="I30" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
-      <c r="F31" t="s">
-        <v>62</v>
-      </c>
-      <c r="G31" t="s">
-        <v>84</v>
-      </c>
-      <c r="H31" t="s">
-        <v>99</v>
-      </c>
       <c r="I31" t="s">
-        <v>125</v>
-      </c>
-      <c r="J31" t="s">
-        <v>161</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" spans="1:10">
-      <c r="A32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" t="s">
-        <v>30</v>
-      </c>
-      <c r="D32" t="s">
-        <v>35</v>
+      <c r="E32" t="s">
+        <v>42</v>
+      </c>
+      <c r="F32" t="s">
+        <v>63</v>
+      </c>
+      <c r="G32" t="s">
+        <v>85</v>
+      </c>
+      <c r="H32" t="s">
+        <v>98</v>
       </c>
       <c r="I32" t="s">
-        <v>126</v>
+        <v>127</v>
+      </c>
+      <c r="J32" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1617,97 +1629,88 @@
         <v>17</v>
       </c>
       <c r="I33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:10">
-      <c r="E34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F34" t="s">
-        <v>63</v>
-      </c>
-      <c r="G34" t="s">
-        <v>85</v>
-      </c>
       <c r="H34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I34" t="s">
-        <v>127</v>
-      </c>
-      <c r="J34" t="s">
-        <v>162</v>
+        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C35" t="s">
+        <v>32</v>
+      </c>
+      <c r="E35" t="s">
+        <v>44</v>
       </c>
       <c r="I35" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:10">
+      <c r="E36" t="s">
+        <v>45</v>
+      </c>
+      <c r="F36" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" t="s">
+        <v>86</v>
+      </c>
       <c r="H36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I36" t="s">
-        <v>128</v>
+        <v>129</v>
+      </c>
+      <c r="J36" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
-        <v>32</v>
-      </c>
-      <c r="E37" t="s">
-        <v>44</v>
+        <v>30</v>
+      </c>
+      <c r="D37" t="s">
+        <v>35</v>
       </c>
       <c r="I37" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:10">
-      <c r="E38" t="s">
-        <v>45</v>
-      </c>
-      <c r="F38" t="s">
-        <v>64</v>
-      </c>
-      <c r="G38" t="s">
-        <v>86</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="A38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
+      <c r="E39" t="s">
+        <v>42</v>
+      </c>
+      <c r="H39" t="s">
         <v>98</v>
       </c>
-      <c r="I38" t="s">
-        <v>129</v>
-      </c>
-      <c r="J38" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10">
-      <c r="A39" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" t="s">
-        <v>23</v>
-      </c>
-      <c r="C39" t="s">
-        <v>30</v>
-      </c>
-      <c r="D39" t="s">
-        <v>35</v>
-      </c>
       <c r="I39" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -1715,29 +1718,50 @@
         <v>17</v>
       </c>
       <c r="I40" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" spans="1:10">
-      <c r="E41" t="s">
-        <v>42</v>
+      <c r="F41" t="s">
+        <v>65</v>
+      </c>
+      <c r="G41" t="s">
+        <v>87</v>
       </c>
       <c r="H41" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I41" t="s">
-        <v>130</v>
+        <v>131</v>
+      </c>
+      <c r="J41" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="B42" t="s">
+        <v>23</v>
+      </c>
+      <c r="C42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D42" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" t="s">
+        <v>42</v>
       </c>
       <c r="I42" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
     </row>
     <row r="43" spans="1:10">
+      <c r="A43" t="s">
+        <v>16</v>
+      </c>
       <c r="F43" t="s">
         <v>65</v>
       </c>
@@ -1745,10 +1769,10 @@
         <v>87</v>
       </c>
       <c r="H43" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="I43" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="J43" t="s">
         <v>164</v>
@@ -1756,42 +1780,39 @@
     </row>
     <row r="44" spans="1:10">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C44" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D44" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I44" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="E45" t="s">
+        <v>46</v>
       </c>
       <c r="F45" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G45" t="s">
-        <v>87</v>
-      </c>
-      <c r="H45" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I45" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="J45" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -1799,16 +1820,13 @@
         <v>18</v>
       </c>
       <c r="B46" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D46" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I46" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -1816,123 +1834,129 @@
         <v>18</v>
       </c>
       <c r="E47" t="s">
-        <v>46</v>
-      </c>
-      <c r="F47" t="s">
-        <v>66</v>
-      </c>
-      <c r="G47" t="s">
-        <v>88</v>
+        <v>47</v>
+      </c>
+      <c r="H47" t="s">
+        <v>95</v>
       </c>
       <c r="I47" t="s">
-        <v>135</v>
-      </c>
-      <c r="J47" t="s">
-        <v>165</v>
+        <v>137</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
-        <v>18</v>
-      </c>
-      <c r="B48" t="s">
-        <v>29</v>
-      </c>
-      <c r="D48" t="s">
-        <v>35</v>
+        <v>19</v>
+      </c>
+      <c r="F48" t="s">
+        <v>67</v>
+      </c>
+      <c r="G48" t="s">
+        <v>89</v>
       </c>
       <c r="I48" t="s">
-        <v>136</v>
+        <v>138</v>
+      </c>
+      <c r="J48" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
         <v>18</v>
       </c>
-      <c r="E49" t="s">
-        <v>47</v>
-      </c>
-      <c r="H49" t="s">
-        <v>95</v>
+      <c r="F49" t="s">
+        <v>68</v>
+      </c>
+      <c r="G49" t="s">
+        <v>90</v>
       </c>
       <c r="I49" t="s">
-        <v>137</v>
+        <v>139</v>
+      </c>
+      <c r="J49" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="A50" t="s">
-        <v>19</v>
-      </c>
-      <c r="F50" t="s">
-        <v>67</v>
-      </c>
-      <c r="G50" t="s">
-        <v>89</v>
+        <v>20</v>
+      </c>
+      <c r="B50" t="s">
+        <v>29</v>
+      </c>
+      <c r="D50" t="s">
+        <v>35</v>
       </c>
       <c r="I50" t="s">
-        <v>138</v>
-      </c>
-      <c r="J50" t="s">
-        <v>166</v>
+        <v>140</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" t="s">
-        <v>18</v>
-      </c>
-      <c r="F51" t="s">
-        <v>68</v>
-      </c>
-      <c r="G51" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="I51" t="s">
-        <v>139</v>
-      </c>
-      <c r="J51" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
     </row>
     <row r="52" spans="1:10">
-      <c r="A52" t="s">
-        <v>20</v>
-      </c>
-      <c r="B52" t="s">
-        <v>29</v>
-      </c>
-      <c r="D52" t="s">
-        <v>35</v>
+      <c r="E52" t="s">
+        <v>42</v>
+      </c>
+      <c r="F52" t="s">
+        <v>69</v>
+      </c>
+      <c r="G52" t="s">
+        <v>91</v>
+      </c>
+      <c r="H52" t="s">
+        <v>98</v>
       </c>
       <c r="I52" t="s">
-        <v>140</v>
+        <v>142</v>
+      </c>
+      <c r="J52" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" t="s">
+        <v>30</v>
+      </c>
+      <c r="D53" t="s">
+        <v>37</v>
+      </c>
+      <c r="F53" t="s">
+        <v>50</v>
       </c>
       <c r="I53" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="E54" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F54" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G54" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H54" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I54" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -1943,112 +1967,72 @@
         <v>28</v>
       </c>
       <c r="C55" t="s">
-        <v>30</v>
-      </c>
-      <c r="D55" t="s">
+        <v>32</v>
+      </c>
+      <c r="E55" t="s">
         <v>37</v>
       </c>
       <c r="F55" t="s">
         <v>50</v>
       </c>
       <c r="I55" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="E56" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F56" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G56" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H56" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I56" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J56" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>28</v>
-      </c>
-      <c r="C57" t="s">
-        <v>32</v>
-      </c>
-      <c r="E57" t="s">
-        <v>37</v>
-      </c>
-      <c r="F57" t="s">
-        <v>50</v>
+        <v>26</v>
+      </c>
+      <c r="D57" t="s">
+        <v>35</v>
       </c>
       <c r="I57" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="58" spans="1:10">
+      <c r="A58" t="s">
+        <v>20</v>
+      </c>
       <c r="E58" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="F58" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G58" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H58" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="I58" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="J58" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10">
-      <c r="A59" t="s">
-        <v>20</v>
-      </c>
-      <c r="B59" t="s">
-        <v>26</v>
-      </c>
-      <c r="D59" t="s">
-        <v>35</v>
-      </c>
-      <c r="I59" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
-      <c r="A60" t="s">
-        <v>20</v>
-      </c>
-      <c r="E60" t="s">
-        <v>41</v>
-      </c>
-      <c r="F60" t="s">
-        <v>72</v>
-      </c>
-      <c r="G60" t="s">
-        <v>94</v>
-      </c>
-      <c r="H60" t="s">
-        <v>95</v>
-      </c>
-      <c r="I60" t="s">
-        <v>148</v>
-      </c>
-      <c r="J60" t="s">
         <v>171</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update fitur logic tgl ro, tgl muat serta perbaikan kualitas akurasi jumlah record output dan input
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="273">
   <si>
     <t>DATE</t>
   </si>
@@ -85,21 +85,48 @@
     <t>12 feb 26</t>
   </si>
   <si>
+    <t>03 : 00 12 februari 2026</t>
+  </si>
+  <si>
+    <t>3 maret 2026</t>
+  </si>
+  <si>
+    <t>03 : 00 04032026</t>
+  </si>
+  <si>
+    <t>03 maret 2026</t>
+  </si>
+  <si>
+    <t>04 maret 2026</t>
+  </si>
+  <si>
+    <t>04 mar 2026</t>
+  </si>
+  <si>
+    <t>05 mar 26</t>
+  </si>
+  <si>
+    <t>05 maret 2026</t>
+  </si>
+  <si>
+    <t>06 maret 2026</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>24</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -115,6 +142,9 @@
     <t>cddl</t>
   </si>
   <si>
+    <t>tronton</t>
+  </si>
+  <si>
     <t>jne</t>
   </si>
   <si>
@@ -130,15 +160,18 @@
     <t>cikarang</t>
   </si>
   <si>
+    <t>cgk sub</t>
+  </si>
+  <si>
+    <t>argo pantes</t>
+  </si>
+  <si>
+    <t>cgk jatim</t>
+  </si>
+  <si>
     <t>subcgk</t>
   </si>
   <si>
-    <t>cgk sub</t>
-  </si>
-  <si>
-    <t>cgk tentatif</t>
-  </si>
-  <si>
     <t>cgk mes</t>
   </si>
   <si>
@@ -166,6 +199,27 @@
     <t>cgkjbr</t>
   </si>
   <si>
+    <t>mes ddriver</t>
+  </si>
+  <si>
+    <t>sub cgk</t>
+  </si>
+  <si>
+    <t>suxcgk</t>
+  </si>
+  <si>
+    <t>cgkpsr</t>
+  </si>
+  <si>
+    <t>jatim tentatif</t>
+  </si>
+  <si>
+    <t>cgksub</t>
+  </si>
+  <si>
+    <t>pku</t>
+  </si>
+  <si>
     <t>akbar</t>
   </si>
   <si>
@@ -235,6 +289,54 @@
     <t>sri mardono</t>
   </si>
   <si>
+    <t>rosyit</t>
+  </si>
+  <si>
+    <t>m . ibnu</t>
+  </si>
+  <si>
+    <t>akiyat</t>
+  </si>
+  <si>
+    <t>ahmad wahyudi</t>
+  </si>
+  <si>
+    <t>ari purnama</t>
+  </si>
+  <si>
+    <t>dedeng</t>
+  </si>
+  <si>
+    <t>jupri</t>
+  </si>
+  <si>
+    <t>andi</t>
+  </si>
+  <si>
+    <t>misno</t>
+  </si>
+  <si>
+    <t>usman afandi</t>
+  </si>
+  <si>
+    <t>miyanta</t>
+  </si>
+  <si>
+    <t>davit</t>
+  </si>
+  <si>
+    <t>iwan hariono</t>
+  </si>
+  <si>
+    <t>suryadi</t>
+  </si>
+  <si>
+    <t>sobar</t>
+  </si>
+  <si>
+    <t>nasip</t>
+  </si>
+  <si>
     <t>n 9549 ua</t>
   </si>
   <si>
@@ -301,6 +403,54 @@
     <t>bk 8678 ve</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>b 9563 teu</t>
+  </si>
+  <si>
+    <t>l 9511 al</t>
+  </si>
+  <si>
+    <t>l 9722 ue</t>
+  </si>
+  <si>
+    <t>w 8323 nv</t>
+  </si>
+  <si>
+    <t>b 9679wt</t>
+  </si>
+  <si>
+    <t>b 9383 txv</t>
+  </si>
+  <si>
+    <t>e 9426 aa</t>
+  </si>
+  <si>
+    <t>bm 9273 ro</t>
+  </si>
+  <si>
+    <t>be 8610 db</t>
+  </si>
+  <si>
+    <t>bn 8038 rp</t>
+  </si>
+  <si>
+    <t>be 8456 fn</t>
+  </si>
+  <si>
+    <t>b 9726 sxw</t>
+  </si>
+  <si>
+    <t>bl 8188 jp</t>
+  </si>
+  <si>
+    <t>l 8183uv</t>
+  </si>
+  <si>
+    <t>bk 8330 vy</t>
+  </si>
+  <si>
     <t>segera</t>
   </si>
   <si>
@@ -314,6 +464,9 @@
   </si>
   <si>
     <t>03 : 00</t>
+  </si>
+  <si>
+    <t>06 : 00</t>
   </si>
   <si>
     <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 06 febuary 2026
@@ -349,16 +502,6 @@
 driver  : Chandra
 Nopol  : L 8601 UH
 No hp  : +62 852-3168-1470</t>
-  </si>
-  <si>
-    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
-06 FEB 2026
-10 UNIT CDDL/24 CBM
-Lokasi : ARGOPANTES</t>
-  </si>
-  <si>
-    <t>Waktu loading : SEGERA
-Rute/tujuan : CGK - JATIM TENTATIF</t>
   </si>
   <si>
     <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCAL
@@ -608,6 +751,299 @@
 No hp  :085218843366</t>
   </si>
   <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 12 FEBRUARI 2026:
+2 unit tronton 50 Cbm
+Lokasi : cikokol</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 12 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+driver  : AGENG
+Nopol  : B 9654 YU
+No hp  : +62 857-0738-0584</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 12 FEBRUARI 2026:
+3 UNIT TWB 50 Cbm
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 12 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+driver  : Rosyit
+Nopol  : B 9563 TEU
+No hp  : 082313572678</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 12 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+driver  : M.ibnu
+Nopol  : L 9511 AL
+No hp  : 082191633212</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00 12 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+driver  : Akiyat
+Nopol  : L 9722 UE
+No hp  :081281122738
+Akbar Rafay: REQUEST ORDER ONCALL 12 FEBRUARI 2026:
+3 UNIT TWB 50 Cbm
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00 12 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+Revisi
+driver  : Ahmad Wahyudi
+Nopol  : W 8323 NV
+No hp  : 085792725002
+Posisi sudah dilokasi muat</t>
+  </si>
+  <si>
+    <t>REQUEST  ORDER  ONCALL  3 MARET 2026
+5 UNIT WB/50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 23:00 3 MARET 2026
+Rute/tujuan : CGK - MES 
+ddriver  : Sri Mardono
+Nopol  : BK 8678 VE
+No hp  : 085218843366</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00 04-03-2026
+Rute/tujuan : CGK - MES 
+driver  :
+Nopol  :
+No hp  :</t>
+  </si>
+  <si>
+    <t>REQUEST  ORDER  ONCALL  3 MARET 2026
+6 UNIT WB/50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 23:00 3 MARET 2026
+Rute/tujuan : CGK - SUB 
+driver  : Rosyit
+Nopol  : B 9562 TEU
+No hp  : 082313572678
+Driver : sofyan
+Nopol : B 9679WT
+No Hp : 082231837381</t>
+  </si>
+  <si>
+    <t>REQUEST  ORDER  ONCALL  3 MARET 2026
+1 UNIT WB/50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 23:00 3 MARET 2026
+Rute/tujuan : SUB - CGK
+driver  : Yuda
+Nopol  : W 8973 UQ
+No hp  : 089507296985</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER ONCALL 03 maret 2026:
+3 unit Cddl 24 Cbm
+Lokasi : Megahub</t>
+  </si>
+  <si>
+    <t>Waktu loading : 23:00 03 maret 2026
+Rute/tujuan : CGK - JATIM
+driver  : Ari purnama
+Nopol  : B 9383 TXV
+No hp : 082136689169
+Fyi pak  @Nomor tidak dikenal@Nomor tidak dikenal</t>
+  </si>
+  <si>
+    <t>REQUEST ULANG ORDER ONCALL 04 MARET 2026:
+8 unit Cddl 24 Cbm
+Lokasi : *argo pantes *</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 04 MARET 2026
+Rute/tujuan : *CGK - Jateng tentatif
+Nama : Dedeng
+Nopol :E 9426 Aa
+No.hp : 0895393659401
+Request Unit On Call Tgl 04 Maret 2026
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 04 Maret 2026
+Rute/tujuan : CGK - PKU
+driver  : Jupri
+Nopol  : BM 9273 RO
+No Hp :082172471454</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER ONCALL
+04 MARET 2026:
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CGK - MES
+driver  : Andi
+Nopol  : BE 8610 DB
+No Hp :081374328877</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CGK - MES
+driver  : Misno
+Nopol  : BN 8038 RP
+No Hp :082211762649</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER ONCALL
+04 MARET 2026:
+REVISI NOPOL BE 8610 DB
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CGK - MES
+driver  : Usman Afandi
+Nopol  : BE 8456 FN
+No Hp : +62 853-7337-2594
+Request Order Oncall  04 Mar 2026
+2 UNIT TWB 50 CBM
+Lokasi : JNE SURABAYA
+Rute/ Tujuan   : SUX-CGK</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 04 Mar 2026
+NAMA   : Wahyudi
+NOPOL : N 9549 UA
+NO HP : 085784422398
+Request Unit On Call Tgl 05 Mar 26
+1 Unit  Cddl / 24 Cbm
+Lokasi : Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : 06:00
+Rute/tujuan : CKR-JBR
+Driver   : miyanta
+Nopol  : F 9647 FH
+No Hp  :08118558105
+Request Unit On Call Tgl 05 Mar 26
+RAFAY
+1 Unit  Cddl / 24 Cbm
+Lokasi : Cikokol + Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00
+Rute/tujuan : CGK-PSR
+Driver   : Davit
+Nopol  : B 9726 SXW
+No Hp  :082117275166</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER ONCALL
+05 MARET 2026:
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 17:00 05-03-2026
+Rute/tujuan : CGK - SUB
+driver  : Iwan Hariono
+Nopol  : BL 8188 JP
+No Hp :081389976421
+Request Order Oncall  05 Maret  2026</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+06 FEB 2026
+10 UNIT CDDL/24 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Rute/tujuan : CGK - JATIM TENTATIF
+2 UNIT TWB 50 CBM
+Lokasi : JNE SURABAYA
+Rute/ Tujuan   : SUX-CGK</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Driver : Akiyat
+Nopol : L 9722 UE
+No HP :081281122738
+REQUER ORDER ULANG DAN TAMBAHAN ON CALL
+06 MARET 2026
+3 UNIT TWB 50 CBM
+ Lokasi : ARGOPANTES
+Rute / tujuan : *JATim TENTATIF</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Nama 	: M. Ibnu
+Nopol		: L 9511 AL
+No Tlp	:082191633212
+Nama : Jamaadi
+Nopol : L 8786 BN
+No Hp :082229973792
+Nama : Suryadi 
+Nopol : L 8183UV
+No hp :085729113217
+REQUER ORDER ULANG DAN TAMBAHAN ON CALL
+06 MARET 2026
+3 UNIT TWB 50 CBM
+ Lokasi : ARGOPANTES
+Rute / tujuan : CGK-SUB</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Nama 	: Yuda
+Nopol		: W 8973 UQ
+No Tlp	:089507296985
+REQUER ORDER ULANG DAN TAMBAHAN ON CALL
+06 MARET 2026
+DATA SUMATERA
+2 UNIT TWB 50 CBM
+ Lokasi : ARGOPANTES
+Rute / tujuan : PKU</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Nama 	: Ridwan
+Nopol		: BK 8330 VY
+No Tlp	: 082382200400
+Fyi pak Sobar data tambahan nya
+REQUER ORDER ULANG DAN TAMBAHAN ON CALL
+06 MARET 2026
+DATA SUMATERA
+2 UNIT TWB 50 CBM
+ Lokasi : ARGOPANTES
+Rute / tujuan : PKU</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Nama 	: Nasip
+Nopol		: BH 8165 QI
+No Tlp	:+6281272463920
+REQUER ORDER ULANG DAN TAMBAHAN ON CALL
+06 MARET 2026
+3 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES
+Rute / tujuan : CGK-SUB</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA
+Nama 	: Wahyudi
+Nopol	: N 9549 UA
+No Tlp	:085784422398</t>
+  </si>
+  <si>
     <t>085784422398</t>
   </si>
   <si>
@@ -675,6 +1111,51 @@
   </si>
   <si>
     <t>085218843366</t>
+  </si>
+  <si>
+    <t>082313572678</t>
+  </si>
+  <si>
+    <t>082191633212</t>
+  </si>
+  <si>
+    <t>081281122738</t>
+  </si>
+  <si>
+    <t>085792725002</t>
+  </si>
+  <si>
+    <t>082136689169</t>
+  </si>
+  <si>
+    <t>0895393659401</t>
+  </si>
+  <si>
+    <t>082172471454</t>
+  </si>
+  <si>
+    <t>081374328877</t>
+  </si>
+  <si>
+    <t>082211762649</t>
+  </si>
+  <si>
+    <t>0 85373372594</t>
+  </si>
+  <si>
+    <t>08118558105</t>
+  </si>
+  <si>
+    <t>082117275166</t>
+  </si>
+  <si>
+    <t>081389976421</t>
+  </si>
+  <si>
+    <t>085729113217</t>
+  </si>
+  <si>
+    <t>082382200400</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1072,19 +1553,19 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I2" t="s">
-        <v>100</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1092,19 +1573,19 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I3" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="J3" t="s">
-        <v>149</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1112,19 +1593,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>100</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1132,22 +1613,22 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="G5" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="H5" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>153</v>
       </c>
       <c r="J5" t="s">
-        <v>150</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1155,72 +1636,81 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="I7" t="s">
-        <v>104</v>
+        <v>155</v>
       </c>
       <c r="J7" t="s">
-        <v>151</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="E8" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="I8" t="s">
-        <v>105</v>
+        <v>156</v>
       </c>
       <c r="J8" t="s">
-        <v>152</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>52</v>
       </c>
       <c r="I9" t="s">
-        <v>106</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="E10" t="s">
-        <v>40</v>
+      <c r="F10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" t="s">
+        <v>110</v>
       </c>
       <c r="H10" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I10" t="s">
-        <v>107</v>
+        <v>158</v>
+      </c>
+      <c r="J10" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1228,36 +1718,39 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>41</v>
+        <v>48</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
       </c>
       <c r="I11" t="s">
-        <v>108</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="F12" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="H12" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I12" t="s">
-        <v>109</v>
+        <v>160</v>
       </c>
       <c r="J12" t="s">
-        <v>153</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1265,335 +1758,323 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I13" t="s">
-        <v>110</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="F14" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="G14" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="H14" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I14" t="s">
-        <v>111</v>
+        <v>161</v>
       </c>
       <c r="J14" t="s">
-        <v>154</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
         <v>12</v>
       </c>
-      <c r="B15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" t="s">
-        <v>30</v>
-      </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="F16" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="H16" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I16" t="s">
-        <v>112</v>
+        <v>163</v>
       </c>
       <c r="J16" t="s">
-        <v>155</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
         <v>12</v>
       </c>
+      <c r="B17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>39</v>
+      </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I17" t="s">
-        <v>113</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="F18" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="G18" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I18" t="s">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="J18" t="s">
-        <v>156</v>
+        <v>243</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="E19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F19" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="I19" t="s">
-        <v>110</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="F20" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s">
-        <v>80</v>
+        <v>115</v>
       </c>
       <c r="H20" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I20" t="s">
-        <v>115</v>
+        <v>166</v>
       </c>
       <c r="J20" t="s">
-        <v>157</v>
+        <v>244</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" t="s">
-        <v>43</v>
+        <v>39</v>
+      </c>
+      <c r="D21" t="s">
+        <v>44</v>
       </c>
       <c r="I21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" t="s">
+        <v>78</v>
+      </c>
+      <c r="G22" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="F22" t="s">
-        <v>59</v>
-      </c>
-      <c r="G22" t="s">
-        <v>81</v>
-      </c>
       <c r="H22" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="I22" t="s">
-        <v>117</v>
+        <v>168</v>
       </c>
       <c r="J22" t="s">
-        <v>158</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
+        <v>41</v>
+      </c>
+      <c r="E23" t="s">
+        <v>55</v>
       </c>
       <c r="I23" t="s">
-        <v>118</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" t="s">
-        <v>14</v>
-      </c>
       <c r="E24" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="G24" t="s">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="H24" t="s">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="I24" t="s">
-        <v>119</v>
+        <v>170</v>
       </c>
       <c r="J24" t="s">
-        <v>159</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" t="s">
-        <v>44</v>
+        <v>39</v>
+      </c>
+      <c r="D25" t="s">
+        <v>45</v>
       </c>
       <c r="I25" t="s">
-        <v>120</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:10">
+      <c r="A26" t="s">
+        <v>16</v>
+      </c>
       <c r="E26" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F26" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="G26" t="s">
-        <v>83</v>
-      </c>
-      <c r="H26" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="I26" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="J26" t="s">
-        <v>160</v>
+        <v>235</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
         <v>16</v>
       </c>
-      <c r="B27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27" t="s">
-        <v>30</v>
-      </c>
-      <c r="D27" t="s">
-        <v>35</v>
+      <c r="F27" t="s">
+        <v>80</v>
+      </c>
+      <c r="G27" t="s">
+        <v>118</v>
       </c>
       <c r="I27" t="s">
-        <v>122</v>
+        <v>173</v>
+      </c>
+      <c r="J27" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" t="s">
         <v>16</v>
       </c>
-      <c r="E28" t="s">
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
         <v>39</v>
       </c>
-      <c r="F28" t="s">
-        <v>51</v>
-      </c>
-      <c r="G28" t="s">
-        <v>73</v>
+      <c r="D28" t="s">
+        <v>45</v>
       </c>
       <c r="I28" t="s">
-        <v>123</v>
-      </c>
-      <c r="J28" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" t="s">
-        <v>16</v>
-      </c>
-      <c r="F29" t="s">
-        <v>62</v>
-      </c>
-      <c r="G29" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="I29" t="s">
-        <v>124</v>
-      </c>
-      <c r="J29" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" spans="1:10">
-      <c r="A30" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" t="s">
-        <v>23</v>
-      </c>
-      <c r="C30" t="s">
-        <v>30</v>
-      </c>
-      <c r="D30" t="s">
-        <v>35</v>
+      <c r="E30" t="s">
+        <v>53</v>
+      </c>
+      <c r="F30" t="s">
+        <v>81</v>
+      </c>
+      <c r="G30" t="s">
+        <v>119</v>
+      </c>
+      <c r="H30" t="s">
+        <v>148</v>
       </c>
       <c r="I30" t="s">
-        <v>125</v>
+        <v>176</v>
+      </c>
+      <c r="J30" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -1601,97 +2082,88 @@
         <v>17</v>
       </c>
       <c r="I31" t="s">
-        <v>126</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:10">
-      <c r="E32" t="s">
-        <v>42</v>
-      </c>
-      <c r="F32" t="s">
-        <v>63</v>
-      </c>
-      <c r="G32" t="s">
-        <v>85</v>
-      </c>
       <c r="H32" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="I32" t="s">
-        <v>127</v>
-      </c>
-      <c r="J32" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="B33" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" t="s">
+        <v>55</v>
       </c>
       <c r="I33" t="s">
-        <v>126</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34" spans="1:10">
+      <c r="E34" t="s">
+        <v>56</v>
+      </c>
+      <c r="F34" t="s">
+        <v>82</v>
+      </c>
+      <c r="G34" t="s">
+        <v>120</v>
+      </c>
       <c r="H34" t="s">
-        <v>99</v>
+        <v>148</v>
       </c>
       <c r="I34" t="s">
-        <v>128</v>
+        <v>178</v>
+      </c>
+      <c r="J34" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
-      </c>
-      <c r="E35" t="s">
-        <v>44</v>
+        <v>39</v>
+      </c>
+      <c r="D35" t="s">
+        <v>45</v>
       </c>
       <c r="I35" t="s">
-        <v>120</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" spans="1:10">
-      <c r="E36" t="s">
-        <v>45</v>
-      </c>
-      <c r="F36" t="s">
-        <v>64</v>
-      </c>
-      <c r="G36" t="s">
-        <v>86</v>
-      </c>
-      <c r="H36" t="s">
-        <v>98</v>
+      <c r="A36" t="s">
+        <v>17</v>
       </c>
       <c r="I36" t="s">
-        <v>129</v>
-      </c>
-      <c r="J36" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37" spans="1:10">
-      <c r="A37" t="s">
-        <v>16</v>
-      </c>
-      <c r="B37" t="s">
-        <v>23</v>
-      </c>
-      <c r="C37" t="s">
-        <v>30</v>
-      </c>
-      <c r="D37" t="s">
-        <v>35</v>
+      <c r="E37" t="s">
+        <v>53</v>
+      </c>
+      <c r="H37" t="s">
+        <v>148</v>
       </c>
       <c r="I37" t="s">
-        <v>125</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -1699,83 +2171,101 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>126</v>
+        <v>175</v>
       </c>
     </row>
     <row r="39" spans="1:10">
-      <c r="E39" t="s">
-        <v>42</v>
+      <c r="F39" t="s">
+        <v>83</v>
+      </c>
+      <c r="G39" t="s">
+        <v>121</v>
       </c>
       <c r="H39" t="s">
-        <v>98</v>
+        <v>149</v>
       </c>
       <c r="I39" t="s">
-        <v>130</v>
+        <v>180</v>
+      </c>
+      <c r="J39" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="B40" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" t="s">
+        <v>39</v>
+      </c>
+      <c r="D40" t="s">
+        <v>45</v>
+      </c>
+      <c r="E40" t="s">
+        <v>53</v>
       </c>
       <c r="I40" t="s">
-        <v>126</v>
+        <v>181</v>
       </c>
     </row>
     <row r="41" spans="1:10">
+      <c r="A41" t="s">
+        <v>16</v>
+      </c>
       <c r="F41" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="G41" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="H41" t="s">
-        <v>99</v>
+        <v>145</v>
       </c>
       <c r="I41" t="s">
-        <v>131</v>
+        <v>182</v>
       </c>
       <c r="J41" t="s">
-        <v>164</v>
+        <v>250</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B42" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="C42" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D42" t="s">
-        <v>35</v>
-      </c>
-      <c r="E42" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I42" t="s">
-        <v>132</v>
+        <v>183</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="E43" t="s">
+        <v>57</v>
       </c>
       <c r="F43" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="G43" t="s">
-        <v>87</v>
-      </c>
-      <c r="H43" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I43" t="s">
-        <v>133</v>
+        <v>184</v>
       </c>
       <c r="J43" t="s">
-        <v>164</v>
+        <v>251</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -1783,16 +2273,13 @@
         <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>28</v>
-      </c>
-      <c r="C44" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D44" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I44" t="s">
-        <v>134</v>
+        <v>185</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -1800,123 +2287,129 @@
         <v>18</v>
       </c>
       <c r="E45" t="s">
-        <v>46</v>
-      </c>
-      <c r="F45" t="s">
-        <v>66</v>
-      </c>
-      <c r="G45" t="s">
-        <v>88</v>
+        <v>58</v>
+      </c>
+      <c r="H45" t="s">
+        <v>145</v>
       </c>
       <c r="I45" t="s">
-        <v>135</v>
-      </c>
-      <c r="J45" t="s">
-        <v>165</v>
+        <v>186</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>18</v>
-      </c>
-      <c r="B46" t="s">
-        <v>29</v>
-      </c>
-      <c r="D46" t="s">
-        <v>35</v>
+        <v>19</v>
+      </c>
+      <c r="F46" t="s">
+        <v>85</v>
+      </c>
+      <c r="G46" t="s">
+        <v>123</v>
       </c>
       <c r="I46" t="s">
-        <v>136</v>
+        <v>187</v>
+      </c>
+      <c r="J46" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
         <v>18</v>
       </c>
-      <c r="E47" t="s">
-        <v>47</v>
-      </c>
-      <c r="H47" t="s">
-        <v>95</v>
+      <c r="F47" t="s">
+        <v>86</v>
+      </c>
+      <c r="G47" t="s">
+        <v>124</v>
       </c>
       <c r="I47" t="s">
-        <v>137</v>
+        <v>188</v>
+      </c>
+      <c r="J47" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
-        <v>19</v>
-      </c>
-      <c r="F48" t="s">
-        <v>67</v>
-      </c>
-      <c r="G48" t="s">
-        <v>89</v>
+        <v>20</v>
+      </c>
+      <c r="B48" t="s">
+        <v>38</v>
+      </c>
+      <c r="D48" t="s">
+        <v>45</v>
       </c>
       <c r="I48" t="s">
-        <v>138</v>
-      </c>
-      <c r="J48" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
-        <v>18</v>
-      </c>
-      <c r="F49" t="s">
-        <v>68</v>
-      </c>
-      <c r="G49" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="I49" t="s">
-        <v>139</v>
-      </c>
-      <c r="J49" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:10">
-      <c r="A50" t="s">
-        <v>20</v>
-      </c>
-      <c r="B50" t="s">
-        <v>29</v>
-      </c>
-      <c r="D50" t="s">
-        <v>35</v>
+      <c r="E50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F50" t="s">
+        <v>87</v>
+      </c>
+      <c r="G50" t="s">
+        <v>125</v>
+      </c>
+      <c r="H50" t="s">
+        <v>148</v>
       </c>
       <c r="I50" t="s">
-        <v>140</v>
+        <v>191</v>
+      </c>
+      <c r="J50" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="B51" t="s">
+        <v>37</v>
+      </c>
+      <c r="C51" t="s">
+        <v>39</v>
+      </c>
+      <c r="D51" t="s">
+        <v>47</v>
+      </c>
+      <c r="F51" t="s">
+        <v>68</v>
       </c>
       <c r="I51" t="s">
-        <v>141</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="E52" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="F52" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="G52" t="s">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="H52" t="s">
-        <v>98</v>
+        <v>145</v>
       </c>
       <c r="I52" t="s">
-        <v>142</v>
+        <v>193</v>
       </c>
       <c r="J52" t="s">
-        <v>168</v>
+        <v>255</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -1924,79 +2417,76 @@
         <v>22</v>
       </c>
       <c r="B53" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C53" t="s">
-        <v>30</v>
-      </c>
-      <c r="D53" t="s">
-        <v>37</v>
+        <v>41</v>
+      </c>
+      <c r="E53" t="s">
+        <v>47</v>
       </c>
       <c r="F53" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="I53" t="s">
-        <v>143</v>
+        <v>194</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="E54" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="F54" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="G54" t="s">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="H54" t="s">
-        <v>95</v>
+        <v>149</v>
       </c>
       <c r="I54" t="s">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="J54" t="s">
-        <v>169</v>
+        <v>256</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>28</v>
-      </c>
-      <c r="C55" t="s">
-        <v>32</v>
-      </c>
-      <c r="E55" t="s">
-        <v>37</v>
-      </c>
-      <c r="F55" t="s">
-        <v>50</v>
+        <v>34</v>
+      </c>
+      <c r="D55" t="s">
+        <v>45</v>
       </c>
       <c r="I55" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
+      <c r="A56" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" t="s">
+        <v>52</v>
+      </c>
+      <c r="F56" t="s">
+        <v>90</v>
+      </c>
+      <c r="G56" t="s">
+        <v>128</v>
+      </c>
+      <c r="H56" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="56" spans="1:10">
-      <c r="E56" t="s">
-        <v>49</v>
-      </c>
-      <c r="F56" t="s">
-        <v>71</v>
-      </c>
-      <c r="G56" t="s">
-        <v>93</v>
-      </c>
-      <c r="H56" t="s">
-        <v>99</v>
-      </c>
       <c r="I56" t="s">
-        <v>146</v>
+        <v>197</v>
       </c>
       <c r="J56" t="s">
-        <v>170</v>
+        <v>257</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2004,13 +2494,16 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>26</v>
+        <v>38</v>
+      </c>
+      <c r="C57" t="s">
+        <v>42</v>
       </c>
       <c r="D57" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="I57" t="s">
-        <v>147</v>
+        <v>198</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2018,22 +2511,840 @@
         <v>20</v>
       </c>
       <c r="E58" t="s">
+        <v>48</v>
+      </c>
+      <c r="F58" t="s">
+        <v>88</v>
+      </c>
+      <c r="G58" t="s">
+        <v>129</v>
+      </c>
+      <c r="H58" t="s">
+        <v>145</v>
+      </c>
+      <c r="I58" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" t="s">
+        <v>34</v>
+      </c>
+      <c r="C59" t="s">
+        <v>39</v>
+      </c>
+      <c r="D59" t="s">
+        <v>44</v>
+      </c>
+      <c r="I59" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" t="s">
+        <v>20</v>
+      </c>
+      <c r="E60" t="s">
+        <v>48</v>
+      </c>
+      <c r="F60" t="s">
+        <v>91</v>
+      </c>
+      <c r="G60" t="s">
+        <v>130</v>
+      </c>
+      <c r="H60" t="s">
+        <v>145</v>
+      </c>
+      <c r="I60" t="s">
+        <v>201</v>
+      </c>
+      <c r="J60" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" t="s">
+        <v>20</v>
+      </c>
+      <c r="E61" t="s">
+        <v>48</v>
+      </c>
+      <c r="F61" t="s">
+        <v>92</v>
+      </c>
+      <c r="G61" t="s">
+        <v>131</v>
+      </c>
+      <c r="H61" t="s">
+        <v>145</v>
+      </c>
+      <c r="I61" t="s">
+        <v>202</v>
+      </c>
+      <c r="J61" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" t="s">
+        <v>20</v>
+      </c>
+      <c r="B62" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" t="s">
+        <v>39</v>
+      </c>
+      <c r="D62" t="s">
+        <v>44</v>
+      </c>
+      <c r="F62" t="s">
+        <v>93</v>
+      </c>
+      <c r="G62" t="s">
+        <v>132</v>
+      </c>
+      <c r="I62" t="s">
+        <v>203</v>
+      </c>
+      <c r="J62" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" t="s">
+        <v>20</v>
+      </c>
+      <c r="E63" t="s">
+        <v>48</v>
+      </c>
+      <c r="F63" t="s">
+        <v>91</v>
+      </c>
+      <c r="G63" t="s">
+        <v>130</v>
+      </c>
+      <c r="H63" t="s">
+        <v>145</v>
+      </c>
+      <c r="I63" t="s">
+        <v>201</v>
+      </c>
+      <c r="J63" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" t="s">
+        <v>20</v>
+      </c>
+      <c r="E64" t="s">
+        <v>48</v>
+      </c>
+      <c r="F64" t="s">
+        <v>92</v>
+      </c>
+      <c r="G64" t="s">
+        <v>131</v>
+      </c>
+      <c r="H64" t="s">
+        <v>145</v>
+      </c>
+      <c r="I64" t="s">
+        <v>202</v>
+      </c>
+      <c r="J64" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
+      <c r="A65" t="s">
+        <v>23</v>
+      </c>
+      <c r="D65" t="s">
+        <v>48</v>
+      </c>
+      <c r="F65" t="s">
+        <v>94</v>
+      </c>
+      <c r="G65" t="s">
+        <v>133</v>
+      </c>
+      <c r="I65" t="s">
+        <v>204</v>
+      </c>
+      <c r="J65" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
+      <c r="A66" t="s">
+        <v>24</v>
+      </c>
+      <c r="B66" t="s">
+        <v>35</v>
+      </c>
+      <c r="C66" t="s">
+        <v>40</v>
+      </c>
+      <c r="D66" t="s">
+        <v>44</v>
+      </c>
+      <c r="I66" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
+      <c r="A67" t="s">
+        <v>24</v>
+      </c>
+      <c r="E67" t="s">
+        <v>61</v>
+      </c>
+      <c r="F67" t="s">
+        <v>90</v>
+      </c>
+      <c r="G67" t="s">
+        <v>128</v>
+      </c>
+      <c r="I67" t="s">
+        <v>206</v>
+      </c>
+      <c r="J67" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" t="s">
+        <v>25</v>
+      </c>
+      <c r="E68" t="s">
+        <v>52</v>
+      </c>
+      <c r="I68" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10">
+      <c r="A69" t="s">
+        <v>24</v>
+      </c>
+      <c r="B69" t="s">
+        <v>33</v>
+      </c>
+      <c r="C69" t="s">
+        <v>40</v>
+      </c>
+      <c r="D69" t="s">
+        <v>44</v>
+      </c>
+      <c r="I69" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10">
+      <c r="A70" t="s">
+        <v>24</v>
+      </c>
+      <c r="E70" t="s">
+        <v>48</v>
+      </c>
+      <c r="F70" t="s">
+        <v>70</v>
+      </c>
+      <c r="G70" t="s">
+        <v>134</v>
+      </c>
+      <c r="I70" t="s">
+        <v>209</v>
+      </c>
+      <c r="J70" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10">
+      <c r="A71" t="s">
+        <v>24</v>
+      </c>
+      <c r="B71" t="s">
+        <v>37</v>
+      </c>
+      <c r="C71" t="s">
+        <v>40</v>
+      </c>
+      <c r="D71" t="s">
+        <v>44</v>
+      </c>
+      <c r="I71" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10">
+      <c r="A72" t="s">
+        <v>24</v>
+      </c>
+      <c r="E72" t="s">
+        <v>62</v>
+      </c>
+      <c r="F72" t="s">
+        <v>80</v>
+      </c>
+      <c r="G72" t="s">
+        <v>118</v>
+      </c>
+      <c r="I72" t="s">
+        <v>211</v>
+      </c>
+      <c r="J72" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10">
+      <c r="A73" t="s">
+        <v>26</v>
+      </c>
+      <c r="B73" t="s">
+        <v>36</v>
+      </c>
+      <c r="C73" t="s">
         <v>41</v>
       </c>
-      <c r="F58" t="s">
-        <v>72</v>
-      </c>
-      <c r="G58" t="s">
-        <v>94</v>
-      </c>
-      <c r="H58" t="s">
+      <c r="D73" t="s">
+        <v>46</v>
+      </c>
+      <c r="I73" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10">
+      <c r="A74" t="s">
+        <v>26</v>
+      </c>
+      <c r="E74" t="s">
+        <v>50</v>
+      </c>
+      <c r="F74" t="s">
         <v>95</v>
       </c>
-      <c r="I58" t="s">
-        <v>148</v>
-      </c>
-      <c r="J58" t="s">
-        <v>171</v>
+      <c r="G74" t="s">
+        <v>135</v>
+      </c>
+      <c r="I74" t="s">
+        <v>213</v>
+      </c>
+      <c r="J74" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10">
+      <c r="A75" t="s">
+        <v>27</v>
+      </c>
+      <c r="B75" t="s">
+        <v>36</v>
+      </c>
+      <c r="C75" t="s">
+        <v>41</v>
+      </c>
+      <c r="D75" t="s">
+        <v>49</v>
+      </c>
+      <c r="I75" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10">
+      <c r="A76" t="s">
+        <v>27</v>
+      </c>
+      <c r="B76" t="s">
+        <v>35</v>
+      </c>
+      <c r="C76" t="s">
+        <v>39</v>
+      </c>
+      <c r="D76" t="s">
+        <v>44</v>
+      </c>
+      <c r="F76" t="s">
+        <v>96</v>
+      </c>
+      <c r="G76" t="s">
+        <v>136</v>
+      </c>
+      <c r="H76" t="s">
+        <v>145</v>
+      </c>
+      <c r="I76" t="s">
+        <v>215</v>
+      </c>
+      <c r="J76" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10">
+      <c r="A77" t="s">
+        <v>27</v>
+      </c>
+      <c r="E77" t="s">
+        <v>53</v>
+      </c>
+      <c r="F77" t="s">
+        <v>97</v>
+      </c>
+      <c r="G77" t="s">
+        <v>137</v>
+      </c>
+      <c r="H77" t="s">
+        <v>145</v>
+      </c>
+      <c r="I77" t="s">
+        <v>216</v>
+      </c>
+      <c r="J77" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10">
+      <c r="A78" t="s">
+        <v>27</v>
+      </c>
+      <c r="B78" t="s">
+        <v>35</v>
+      </c>
+      <c r="C78" t="s">
+        <v>39</v>
+      </c>
+      <c r="D78" t="s">
+        <v>44</v>
+      </c>
+      <c r="I78" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10">
+      <c r="E79" t="s">
+        <v>52</v>
+      </c>
+      <c r="F79" t="s">
+        <v>98</v>
+      </c>
+      <c r="G79" t="s">
+        <v>138</v>
+      </c>
+      <c r="H79" t="s">
+        <v>145</v>
+      </c>
+      <c r="I79" t="s">
+        <v>218</v>
+      </c>
+      <c r="J79" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10">
+      <c r="E80" t="s">
+        <v>52</v>
+      </c>
+      <c r="F80" t="s">
+        <v>99</v>
+      </c>
+      <c r="G80" t="s">
+        <v>139</v>
+      </c>
+      <c r="H80" t="s">
+        <v>145</v>
+      </c>
+      <c r="I80" t="s">
+        <v>219</v>
+      </c>
+      <c r="J80" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10">
+      <c r="A81" t="s">
+        <v>27</v>
+      </c>
+      <c r="B81" t="s">
+        <v>35</v>
+      </c>
+      <c r="C81" t="s">
+        <v>39</v>
+      </c>
+      <c r="D81" t="s">
+        <v>44</v>
+      </c>
+      <c r="G81" t="s">
+        <v>138</v>
+      </c>
+      <c r="I81" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10">
+      <c r="A82" t="s">
+        <v>28</v>
+      </c>
+      <c r="B82" t="s">
+        <v>32</v>
+      </c>
+      <c r="C82" t="s">
+        <v>39</v>
+      </c>
+      <c r="E82" t="s">
+        <v>63</v>
+      </c>
+      <c r="F82" t="s">
+        <v>100</v>
+      </c>
+      <c r="G82" t="s">
+        <v>140</v>
+      </c>
+      <c r="H82" t="s">
+        <v>145</v>
+      </c>
+      <c r="I82" t="s">
+        <v>221</v>
+      </c>
+      <c r="J82" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10">
+      <c r="A83" t="s">
+        <v>29</v>
+      </c>
+      <c r="B83" t="s">
+        <v>37</v>
+      </c>
+      <c r="C83" t="s">
+        <v>41</v>
+      </c>
+      <c r="E83" t="s">
+        <v>47</v>
+      </c>
+      <c r="F83" t="s">
+        <v>69</v>
+      </c>
+      <c r="G83" t="s">
+        <v>107</v>
+      </c>
+      <c r="H83" t="s">
+        <v>145</v>
+      </c>
+      <c r="I83" t="s">
+        <v>222</v>
+      </c>
+      <c r="J83" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10">
+      <c r="A84" t="s">
+        <v>29</v>
+      </c>
+      <c r="B84" t="s">
+        <v>37</v>
+      </c>
+      <c r="C84" t="s">
+        <v>41</v>
+      </c>
+      <c r="D84" t="s">
+        <v>45</v>
+      </c>
+      <c r="E84" t="s">
+        <v>47</v>
+      </c>
+      <c r="F84" t="s">
+        <v>101</v>
+      </c>
+      <c r="G84" t="s">
+        <v>127</v>
+      </c>
+      <c r="H84" t="s">
+        <v>150</v>
+      </c>
+      <c r="I84" t="s">
+        <v>223</v>
+      </c>
+      <c r="J84" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10">
+      <c r="E85" t="s">
+        <v>64</v>
+      </c>
+      <c r="F85" t="s">
+        <v>102</v>
+      </c>
+      <c r="G85" t="s">
+        <v>141</v>
+      </c>
+      <c r="H85" t="s">
+        <v>149</v>
+      </c>
+      <c r="I85" t="s">
+        <v>224</v>
+      </c>
+      <c r="J85" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10">
+      <c r="A86" t="s">
+        <v>30</v>
+      </c>
+      <c r="B86" t="s">
+        <v>35</v>
+      </c>
+      <c r="C86" t="s">
+        <v>39</v>
+      </c>
+      <c r="D86" t="s">
+        <v>44</v>
+      </c>
+      <c r="I86" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10">
+      <c r="A87" t="s">
+        <v>30</v>
+      </c>
+      <c r="E87" t="s">
+        <v>48</v>
+      </c>
+      <c r="F87" t="s">
+        <v>103</v>
+      </c>
+      <c r="G87" t="s">
+        <v>142</v>
+      </c>
+      <c r="I87" t="s">
+        <v>226</v>
+      </c>
+      <c r="J87" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10">
+      <c r="A88" t="s">
+        <v>11</v>
+      </c>
+      <c r="B88" t="s">
+        <v>36</v>
+      </c>
+      <c r="C88" t="s">
+        <v>41</v>
+      </c>
+      <c r="D88" t="s">
+        <v>44</v>
+      </c>
+      <c r="I88" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10">
+      <c r="B89" t="s">
+        <v>32</v>
+      </c>
+      <c r="C89" t="s">
+        <v>39</v>
+      </c>
+      <c r="D89" t="s">
+        <v>50</v>
+      </c>
+      <c r="E89" t="s">
+        <v>63</v>
+      </c>
+      <c r="H89" t="s">
+        <v>145</v>
+      </c>
+      <c r="I89" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10">
+      <c r="A90" t="s">
+        <v>31</v>
+      </c>
+      <c r="B90" t="s">
+        <v>34</v>
+      </c>
+      <c r="C90" t="s">
+        <v>39</v>
+      </c>
+      <c r="D90" t="s">
+        <v>44</v>
+      </c>
+      <c r="E90" t="s">
+        <v>65</v>
+      </c>
+      <c r="F90" t="s">
+        <v>93</v>
+      </c>
+      <c r="G90" t="s">
+        <v>132</v>
+      </c>
+      <c r="H90" t="s">
+        <v>145</v>
+      </c>
+      <c r="I90" t="s">
+        <v>229</v>
+      </c>
+      <c r="J90" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10">
+      <c r="A91" t="s">
+        <v>31</v>
+      </c>
+      <c r="B91" t="s">
+        <v>34</v>
+      </c>
+      <c r="C91" t="s">
+        <v>39</v>
+      </c>
+      <c r="D91" t="s">
+        <v>44</v>
+      </c>
+      <c r="E91" t="s">
+        <v>66</v>
+      </c>
+      <c r="F91" t="s">
+        <v>104</v>
+      </c>
+      <c r="G91" t="s">
+        <v>143</v>
+      </c>
+      <c r="H91" t="s">
+        <v>145</v>
+      </c>
+      <c r="I91" t="s">
+        <v>230</v>
+      </c>
+      <c r="J91" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10">
+      <c r="A92" t="s">
+        <v>31</v>
+      </c>
+      <c r="B92" t="s">
+        <v>32</v>
+      </c>
+      <c r="C92" t="s">
+        <v>39</v>
+      </c>
+      <c r="D92" t="s">
+        <v>44</v>
+      </c>
+      <c r="E92" t="s">
+        <v>67</v>
+      </c>
+      <c r="F92" t="s">
+        <v>80</v>
+      </c>
+      <c r="G92" t="s">
+        <v>118</v>
+      </c>
+      <c r="H92" t="s">
+        <v>145</v>
+      </c>
+      <c r="I92" t="s">
+        <v>231</v>
+      </c>
+      <c r="J92" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10">
+      <c r="A93" t="s">
+        <v>31</v>
+      </c>
+      <c r="B93" t="s">
+        <v>32</v>
+      </c>
+      <c r="C93" t="s">
+        <v>39</v>
+      </c>
+      <c r="D93" t="s">
+        <v>44</v>
+      </c>
+      <c r="E93" t="s">
+        <v>67</v>
+      </c>
+      <c r="F93" t="s">
+        <v>105</v>
+      </c>
+      <c r="G93" t="s">
+        <v>144</v>
+      </c>
+      <c r="H93" t="s">
+        <v>145</v>
+      </c>
+      <c r="I93" t="s">
+        <v>232</v>
+      </c>
+      <c r="J93" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10">
+      <c r="A94" t="s">
+        <v>31</v>
+      </c>
+      <c r="B94" t="s">
+        <v>34</v>
+      </c>
+      <c r="C94" t="s">
+        <v>39</v>
+      </c>
+      <c r="D94" t="s">
+        <v>44</v>
+      </c>
+      <c r="E94" t="s">
+        <v>66</v>
+      </c>
+      <c r="F94" t="s">
+        <v>106</v>
+      </c>
+      <c r="G94" t="s">
+        <v>125</v>
+      </c>
+      <c r="H94" t="s">
+        <v>145</v>
+      </c>
+      <c r="I94" t="s">
+        <v>233</v>
+      </c>
+      <c r="J94" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10">
+      <c r="F95" t="s">
+        <v>69</v>
+      </c>
+      <c r="G95" t="s">
+        <v>107</v>
+      </c>
+      <c r="H95" t="s">
+        <v>145</v>
+      </c>
+      <c r="I95" t="s">
+        <v>234</v>
+      </c>
+      <c r="J95" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perbaikan revisi logic tgl ro dan tgl muat sesuai logika logistik yang benar
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="278">
   <si>
     <t>DATE</t>
   </si>
@@ -112,6 +112,9 @@
     <t>06 maret 2026</t>
   </si>
   <si>
+    <t>18 : 00 05022026</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -337,6 +340,9 @@
     <t>nasip</t>
   </si>
   <si>
+    <t>syarial</t>
+  </si>
+  <si>
     <t>n 9549 ua</t>
   </si>
   <si>
@@ -449,6 +455,9 @@
   </si>
   <si>
     <t>bk 8330 vy</t>
+  </si>
+  <si>
+    <t>bm 8486 au</t>
   </si>
   <si>
     <t>segera</t>
@@ -1034,14 +1043,23 @@
 REQUER ORDER ULANG DAN TAMBAHAN ON CALL
 06 MARET 2026
 3 UNIT TWB 50 CBM
-Lokasi : ARGOPANTES
+ Lokasi : ARGOPANTES
 Rute / tujuan : CGK-SUB</t>
   </si>
   <si>
     <t>Waktu loading : SEGERA
 Nama 	: Wahyudi
-Nopol	: N 9549 UA
-No Tlp	:085784422398</t>
+Nopol		: N 9549 UA
+No Tlp	:085784422398
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES</t>
+  </si>
+  <si>
+    <t>Waktu loading : 18:00 05-02-2026
+Rute/tujuan : CGK - PKU
+driver  : Syarial
+Nopol  :BM 8486 AU
+No Hp :081317708658</t>
   </si>
   <si>
     <t>085784422398</t>
@@ -1156,6 +1174,9 @@
   </si>
   <si>
     <t>082382200400</t>
+  </si>
+  <si>
+    <t>081317708658</t>
   </si>
 </sst>
 </file>
@@ -1513,7 +1534,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1553,19 +1574,19 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1573,19 +1594,19 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1593,19 +1614,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1613,22 +1634,22 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J5" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1636,44 +1657,44 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="I7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J7" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="E8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J8" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1681,36 +1702,36 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I9" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="F10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H10" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I10" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="J10" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1718,39 +1739,39 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="F12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I12" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="J12" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1758,39 +1779,39 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I13" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="F14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G14" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H14" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I14" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J14" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1798,33 +1819,33 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I15" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="F16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H16" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I16" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J16" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1832,39 +1853,39 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="F18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H18" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I18" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="J18" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1872,33 +1893,33 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I19" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="F20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H20" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I20" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="J20" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1906,16 +1927,16 @@
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I21" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1923,22 +1944,22 @@
         <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H22" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I22" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="J22" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1946,36 +1967,36 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I23" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="E24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I24" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="J24" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1983,16 +2004,16 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I25" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2000,19 +2021,19 @@
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G26" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I26" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J26" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2020,16 +2041,16 @@
         <v>16</v>
       </c>
       <c r="F27" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I27" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J27" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2037,16 +2058,16 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I28" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -2054,27 +2075,27 @@
         <v>17</v>
       </c>
       <c r="I29" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="E30" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G30" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H30" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I30" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="J30" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -2082,15 +2103,15 @@
         <v>17</v>
       </c>
       <c r="I31" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="H32" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I32" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -2098,36 +2119,36 @@
         <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E33" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I33" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:10">
       <c r="E34" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F34" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H34" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I34" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J34" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -2135,16 +2156,16 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D35" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I35" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -2152,18 +2173,18 @@
         <v>17</v>
       </c>
       <c r="I36" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="E37" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H37" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I37" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2171,24 +2192,24 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="F39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G39" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H39" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I39" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="J39" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2196,19 +2217,19 @@
         <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C40" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E40" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I40" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2216,19 +2237,19 @@
         <v>16</v>
       </c>
       <c r="F41" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G41" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H41" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I41" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="J41" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -2236,16 +2257,16 @@
         <v>18</v>
       </c>
       <c r="B42" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C42" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D42" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I42" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -2253,19 +2274,19 @@
         <v>18</v>
       </c>
       <c r="E43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F43" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G43" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I43" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="J43" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -2273,13 +2294,13 @@
         <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D44" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I44" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -2287,13 +2308,13 @@
         <v>18</v>
       </c>
       <c r="E45" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H45" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I45" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -2301,16 +2322,16 @@
         <v>19</v>
       </c>
       <c r="F46" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G46" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I46" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="J46" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -2318,16 +2339,16 @@
         <v>18</v>
       </c>
       <c r="F47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G47" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I47" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="J47" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -2335,13 +2356,13 @@
         <v>20</v>
       </c>
       <c r="B48" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D48" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I48" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -2349,27 +2370,27 @@
         <v>21</v>
       </c>
       <c r="I49" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="E50" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F50" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G50" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H50" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I50" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="J50" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -2377,39 +2398,39 @@
         <v>22</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D51" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F51" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I51" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="52" spans="1:10">
       <c r="E52" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F52" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G52" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H52" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I52" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="J52" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -2417,39 +2438,39 @@
         <v>22</v>
       </c>
       <c r="B53" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C53" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E53" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F53" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I53" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="E54" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F54" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G54" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H54" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I54" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="J54" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -2457,13 +2478,13 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D55" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I55" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -2471,22 +2492,22 @@
         <v>20</v>
       </c>
       <c r="E56" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G56" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H56" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I56" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J56" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2494,16 +2515,16 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D57" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I57" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2511,19 +2532,19 @@
         <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F58" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G58" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H58" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I58" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -2531,16 +2552,16 @@
         <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C59" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D59" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I59" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -2548,22 +2569,22 @@
         <v>20</v>
       </c>
       <c r="E60" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F60" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G60" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H60" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I60" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="J60" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -2571,22 +2592,22 @@
         <v>20</v>
       </c>
       <c r="E61" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F61" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H61" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I61" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="J61" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -2594,25 +2615,25 @@
         <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C62" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D62" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F62" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G62" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I62" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="J62" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -2620,22 +2641,22 @@
         <v>20</v>
       </c>
       <c r="E63" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F63" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G63" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H63" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I63" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="J63" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -2643,22 +2664,22 @@
         <v>20</v>
       </c>
       <c r="E64" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G64" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H64" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I64" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="J64" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -2666,19 +2687,19 @@
         <v>23</v>
       </c>
       <c r="D65" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F65" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G65" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I65" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="J65" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -2686,16 +2707,16 @@
         <v>24</v>
       </c>
       <c r="B66" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C66" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D66" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I66" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -2703,19 +2724,19 @@
         <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G67" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I67" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J67" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -2723,10 +2744,10 @@
         <v>25</v>
       </c>
       <c r="E68" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I68" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -2734,16 +2755,16 @@
         <v>24</v>
       </c>
       <c r="B69" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C69" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D69" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I69" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -2751,19 +2772,19 @@
         <v>24</v>
       </c>
       <c r="E70" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F70" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G70" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I70" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="J70" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="71" spans="1:10">
@@ -2771,16 +2792,16 @@
         <v>24</v>
       </c>
       <c r="B71" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C71" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D71" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I71" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="72" spans="1:10">
@@ -2788,19 +2809,19 @@
         <v>24</v>
       </c>
       <c r="E72" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F72" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G72" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I72" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="J72" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="73" spans="1:10">
@@ -2808,16 +2829,16 @@
         <v>26</v>
       </c>
       <c r="B73" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C73" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D73" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I73" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="74" spans="1:10">
@@ -2825,19 +2846,19 @@
         <v>26</v>
       </c>
       <c r="E74" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F74" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G74" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I74" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="J74" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="75" spans="1:10">
@@ -2845,16 +2866,16 @@
         <v>27</v>
       </c>
       <c r="B75" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C75" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D75" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I75" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="76" spans="1:10">
@@ -2862,28 +2883,28 @@
         <v>27</v>
       </c>
       <c r="B76" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C76" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D76" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F76" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G76" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H76" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I76" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="J76" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="77" spans="1:10">
@@ -2891,22 +2912,22 @@
         <v>27</v>
       </c>
       <c r="E77" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F77" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G77" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H77" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I77" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="J77" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="78" spans="1:10">
@@ -2914,56 +2935,56 @@
         <v>27</v>
       </c>
       <c r="B78" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C78" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I78" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="E79" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F79" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G79" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H79" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I79" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="J79" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="E80" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F80" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G80" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H80" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I80" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="J80" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="81" spans="1:10">
@@ -2971,19 +2992,19 @@
         <v>27</v>
       </c>
       <c r="B81" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C81" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D81" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G81" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I81" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="82" spans="1:10">
@@ -2991,28 +3012,28 @@
         <v>28</v>
       </c>
       <c r="B82" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C82" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E82" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F82" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G82" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H82" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I82" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="J82" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="83" spans="1:10">
@@ -3020,28 +3041,28 @@
         <v>29</v>
       </c>
       <c r="B83" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C83" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E83" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F83" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G83" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H83" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I83" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="J83" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="84" spans="1:10">
@@ -3049,51 +3070,51 @@
         <v>29</v>
       </c>
       <c r="B84" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C84" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D84" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E84" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F84" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G84" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H84" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I84" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J84" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="85" spans="1:10">
       <c r="E85" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F85" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G85" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H85" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I85" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="J85" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -3101,16 +3122,16 @@
         <v>30</v>
       </c>
       <c r="B86" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C86" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D86" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I86" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="87" spans="1:10">
@@ -3118,19 +3139,19 @@
         <v>30</v>
       </c>
       <c r="E87" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F87" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G87" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I87" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="J87" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="88" spans="1:10">
@@ -3138,36 +3159,36 @@
         <v>11</v>
       </c>
       <c r="B88" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C88" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D88" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I88" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="89" spans="1:10">
       <c r="B89" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C89" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D89" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E89" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H89" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I89" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="90" spans="1:10">
@@ -3175,31 +3196,31 @@
         <v>31</v>
       </c>
       <c r="B90" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C90" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D90" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E90" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F90" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G90" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H90" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I90" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="J90" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="91" spans="1:10">
@@ -3207,31 +3228,31 @@
         <v>31</v>
       </c>
       <c r="B91" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C91" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D91" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E91" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F91" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G91" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H91" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I91" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="J91" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="92" spans="1:10">
@@ -3239,31 +3260,31 @@
         <v>31</v>
       </c>
       <c r="B92" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C92" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D92" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E92" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F92" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G92" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H92" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I92" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="J92" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="93" spans="1:10">
@@ -3271,31 +3292,31 @@
         <v>31</v>
       </c>
       <c r="B93" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C93" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D93" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E93" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F93" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G93" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H93" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I93" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="J93" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
     </row>
     <row r="94" spans="1:10">
@@ -3303,48 +3324,77 @@
         <v>31</v>
       </c>
       <c r="B94" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C94" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D94" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E94" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F94" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G94" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H94" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I94" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="J94" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="95" spans="1:10">
+      <c r="B95" t="s">
+        <v>36</v>
+      </c>
+      <c r="C95" t="s">
+        <v>40</v>
+      </c>
+      <c r="D95" t="s">
+        <v>45</v>
+      </c>
       <c r="F95" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G95" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H95" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I95" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J95" t="s">
-        <v>235</v>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10">
+      <c r="A96" t="s">
+        <v>32</v>
+      </c>
+      <c r="E96" t="s">
+        <v>54</v>
+      </c>
+      <c r="F96" t="s">
+        <v>108</v>
+      </c>
+      <c r="G96" t="s">
+        <v>147</v>
+      </c>
+      <c r="I96" t="s">
+        <v>238</v>
+      </c>
+      <c r="J96" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update perbaikan logika tgl ro dan tgl muat
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="282">
   <si>
     <t>DATE</t>
   </si>
@@ -70,6 +70,9 @@
     <t>10 / 02 / 2026</t>
   </si>
   <si>
+    <t>02 . 00 / 10</t>
+  </si>
+  <si>
     <t>11 februari 2026</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>3 maret 2026</t>
   </si>
   <si>
-    <t>03 : 00 04032026</t>
+    <t>03 : 00 / 04</t>
   </si>
   <si>
     <t>03 maret 2026</t>
@@ -106,13 +109,16 @@
     <t>05 mar 26</t>
   </si>
   <si>
+    <t>06 mar 26</t>
+  </si>
+  <si>
     <t>05 maret 2026</t>
   </si>
   <si>
     <t>06 maret 2026</t>
   </si>
   <si>
-    <t>18 : 00 05022026</t>
+    <t>18 : 00 / 05</t>
   </si>
   <si>
     <t>2</t>
@@ -643,7 +649,7 @@
 NO HP :</t>
   </si>
   <si>
-    <t>Waktu loading : 02:00
+    <t>Waktu loading :  02.00/10
 Rute/tujuan : SRG-CGK
 Driver : Supriadi
 Nopol : B 9586 TXV
@@ -726,7 +732,7 @@
 Lokasi : Cikarang</t>
   </si>
   <si>
-    <t>Waktu loading : SEGERA
+    <t>Waktu loading : SEGERA 12 Feb 26
 Rute/tujuan : CKR-SUB-SUX 
 Driver   : AGENG
 Nopol  : B9654YU
@@ -822,7 +828,7 @@
 No hp  : 085218843366</t>
   </si>
   <si>
-    <t>Waktu loading : 03:00 04-03-2026
+    <t>Waktu loading :  03:00/04
 Rute/tujuan : CGK - MES 
 driver  :
 Nopol  :
@@ -938,6 +944,9 @@
 Lokasi : Cikarang</t>
   </si>
   <si>
+    <t>REQUEST ORDER KHUSUS 06 Mar 26</t>
+  </si>
+  <si>
     <t>Waktu loading : 06:00
 Rute/tujuan : CKR-JBR
 Driver   : miyanta
@@ -949,6 +958,9 @@
 Lokasi : Cikokol + Cikarang</t>
   </si>
   <si>
+    <t>REQUEST ORDER KHUSUS 06  Mar 26</t>
+  </si>
+  <si>
     <t>Waktu loading : 03:00
 Rute/tujuan : CGK-PSR
 Driver   : Davit
@@ -962,7 +974,7 @@
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading : 17:00 05-03-2026
+    <t>Waktu loading :  17:00/05
 Rute/tujuan : CGK - SUB
 driver  : Iwan Hariono
 Nopol  : BL 8188 JP
@@ -1055,7 +1067,7 @@
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading : 18:00 05-02-2026
+    <t>Waktu loading :  18:00/05
 Rute/tujuan : CGK - PKU
 driver  : Syarial
 Nopol  :BM 8486 AU
@@ -1534,7 +1546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1574,19 +1586,19 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1594,19 +1606,19 @@
         <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="J3" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1614,19 +1626,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1634,22 +1646,22 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="J5" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1657,44 +1669,44 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="I7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J7" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="E8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I8" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J8" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1702,36 +1714,36 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="F10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="J10" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1739,39 +1751,39 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="F12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="J12" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1779,39 +1791,39 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I13" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="F14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G14" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I14" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J14" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1819,33 +1831,33 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="F16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="J16" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1853,39 +1865,39 @@
         <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I17" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="F18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G18" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H18" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I18" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J18" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1893,33 +1905,33 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I19" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="F20" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H20" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I20" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="J20" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1927,16 +1939,16 @@
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I21" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1944,22 +1956,22 @@
         <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H22" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I22" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J22" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1967,36 +1979,36 @@
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I23" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="E24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H24" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I24" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J24" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2004,16 +2016,16 @@
         <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I25" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2021,19 +2033,19 @@
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G26" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I26" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J26" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2041,16 +2053,16 @@
         <v>16</v>
       </c>
       <c r="F27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G27" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I27" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J27" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2058,16 +2070,16 @@
         <v>16</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D28" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I28" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -2075,27 +2087,27 @@
         <v>17</v>
       </c>
       <c r="I29" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="E30" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G30" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H30" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I30" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J30" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -2103,15 +2115,15 @@
         <v>17</v>
       </c>
       <c r="I31" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="H32" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I32" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -2119,36 +2131,36 @@
         <v>15</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C33" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E33" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I33" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" spans="1:10">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
       <c r="E34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G34" t="s">
-        <v>122</v>
-      </c>
-      <c r="H34" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="I34" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J34" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -2156,16 +2168,16 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I35" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -2173,18 +2185,18 @@
         <v>17</v>
       </c>
       <c r="I36" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="E37" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H37" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I37" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2192,24 +2204,24 @@
         <v>17</v>
       </c>
       <c r="I38" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="F39" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G39" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H39" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I39" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J39" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2217,19 +2229,19 @@
         <v>16</v>
       </c>
       <c r="B40" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D40" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E40" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I40" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2237,1164 +2249,1183 @@
         <v>16</v>
       </c>
       <c r="F41" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G41" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H41" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I41" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J41" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B42" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D42" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I42" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E43" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F43" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G43" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I43" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J43" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="44" spans="1:10">
       <c r="A44" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B44" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D44" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I44" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E45" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H45" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I45" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F46" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G46" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I46" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J46" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F47" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G47" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I47" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="J47" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:10">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B48" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D48" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I48" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49" spans="1:10">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I49" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:10">
       <c r="E50" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F50" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G50" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H50" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I50" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J50" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="51" spans="1:10">
       <c r="A51" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D51" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F51" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I51" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="52" spans="1:10">
+      <c r="A52" t="s">
+        <v>23</v>
+      </c>
       <c r="E52" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F52" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G52" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H52" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I52" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J52" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="53" spans="1:10">
       <c r="A53" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E53" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F53" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I53" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="54" spans="1:10">
       <c r="E54" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F54" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G54" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H54" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I54" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J54" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="55" spans="1:10">
       <c r="A55" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B55" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D55" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I55" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="56" spans="1:10">
       <c r="A56" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F56" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G56" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H56" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I56" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="J56" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57" spans="1:10">
       <c r="A57" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C57" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D57" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I57" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="58" spans="1:10">
       <c r="A58" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E58" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F58" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G58" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H58" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I58" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="59" spans="1:10">
       <c r="A59" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B59" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C59" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D59" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I59" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="60" spans="1:10">
       <c r="A60" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E60" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F60" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G60" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H60" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I60" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J60" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="61" spans="1:10">
       <c r="A61" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E61" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F61" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G61" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H61" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I61" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J61" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="62" spans="1:10">
       <c r="A62" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B62" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C62" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D62" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F62" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G62" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I62" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J62" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="63" spans="1:10">
       <c r="A63" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E63" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F63" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G63" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H63" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I63" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J63" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="64" spans="1:10">
       <c r="A64" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E64" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F64" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G64" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H64" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I64" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J64" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="65" spans="1:10">
       <c r="A65" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D65" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F65" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G65" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I65" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="J65" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B66" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C66" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D66" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I66" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:10">
       <c r="A67" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E67" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F67" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G67" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I67" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J67" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="68" spans="1:10">
       <c r="A68" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E68" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I68" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" spans="1:10">
       <c r="A69" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B69" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C69" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D69" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I69" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E70" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F70" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G70" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I70" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J70" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="71" spans="1:10">
       <c r="A71" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B71" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D71" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I71" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="72" spans="1:10">
       <c r="A72" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E72" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F72" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G72" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I72" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J72" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="73" spans="1:10">
       <c r="A73" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B73" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D73" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I73" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E74" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F74" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G74" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I74" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J74" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
     </row>
     <row r="75" spans="1:10">
       <c r="A75" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B75" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C75" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D75" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I75" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="76" spans="1:10">
       <c r="A76" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B76" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C76" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D76" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F76" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="G76" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H76" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I76" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J76" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="77" spans="1:10">
       <c r="A77" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E77" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F77" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G77" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H77" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I77" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="J77" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="78" spans="1:10">
       <c r="A78" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B78" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C78" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D78" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I78" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="79" spans="1:10">
       <c r="E79" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F79" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G79" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H79" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I79" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J79" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="80" spans="1:10">
       <c r="E80" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F80" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G80" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H80" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I80" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J80" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="81" spans="1:10">
       <c r="A81" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B81" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C81" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D81" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G81" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I81" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="82" spans="1:10">
       <c r="A82" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B82" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C82" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E82" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F82" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G82" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H82" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I82" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="J82" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="83" spans="1:10">
       <c r="A83" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B83" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C83" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E83" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F83" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G83" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H83" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I83" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="J83" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" t="s">
-        <v>29</v>
-      </c>
-      <c r="B84" t="s">
-        <v>38</v>
-      </c>
-      <c r="C84" t="s">
-        <v>42</v>
-      </c>
-      <c r="D84" t="s">
-        <v>46</v>
-      </c>
-      <c r="E84" t="s">
+        <v>31</v>
+      </c>
+      <c r="I84" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10">
+      <c r="A85" t="s">
+        <v>30</v>
+      </c>
+      <c r="B85" t="s">
+        <v>40</v>
+      </c>
+      <c r="C85" t="s">
+        <v>44</v>
+      </c>
+      <c r="D85" t="s">
         <v>48</v>
       </c>
-      <c r="F84" t="s">
-        <v>102</v>
-      </c>
-      <c r="G84" t="s">
-        <v>129</v>
-      </c>
-      <c r="H84" t="s">
-        <v>153</v>
-      </c>
-      <c r="I84" t="s">
-        <v>226</v>
-      </c>
-      <c r="J84" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10">
       <c r="E85" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="F85" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G85" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="H85" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I85" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="J85" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="86" spans="1:10">
       <c r="A86" t="s">
-        <v>30</v>
-      </c>
-      <c r="B86" t="s">
-        <v>36</v>
-      </c>
-      <c r="C86" t="s">
-        <v>40</v>
-      </c>
-      <c r="D86" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="I86" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="87" spans="1:10">
-      <c r="A87" t="s">
-        <v>30</v>
-      </c>
       <c r="E87" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="F87" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G87" t="s">
-        <v>144</v>
+        <v>145</v>
+      </c>
+      <c r="H87" t="s">
+        <v>154</v>
       </c>
       <c r="I87" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="J87" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="B88" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C88" t="s">
         <v>42</v>
       </c>
       <c r="D88" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I88" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89" spans="1:10">
-      <c r="B89" t="s">
-        <v>33</v>
-      </c>
-      <c r="C89" t="s">
-        <v>40</v>
-      </c>
-      <c r="D89" t="s">
+      <c r="A89" t="s">
+        <v>32</v>
+      </c>
+      <c r="E89" t="s">
         <v>51</v>
       </c>
-      <c r="E89" t="s">
-        <v>64</v>
-      </c>
-      <c r="H89" t="s">
-        <v>148</v>
+      <c r="F89" t="s">
+        <v>106</v>
+      </c>
+      <c r="G89" t="s">
+        <v>146</v>
       </c>
       <c r="I89" t="s">
-        <v>231</v>
+        <v>233</v>
+      </c>
+      <c r="J89" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="B90" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C90" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D90" t="s">
-        <v>45</v>
-      </c>
-      <c r="E90" t="s">
-        <v>66</v>
-      </c>
-      <c r="F90" t="s">
-        <v>94</v>
-      </c>
-      <c r="G90" t="s">
-        <v>134</v>
-      </c>
-      <c r="H90" t="s">
-        <v>148</v>
+        <v>47</v>
       </c>
       <c r="I90" t="s">
-        <v>232</v>
-      </c>
-      <c r="J90" t="s">
-        <v>264</v>
+        <v>234</v>
       </c>
     </row>
     <row r="91" spans="1:10">
-      <c r="A91" t="s">
-        <v>31</v>
-      </c>
       <c r="B91" t="s">
         <v>35</v>
       </c>
       <c r="C91" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D91" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="E91" t="s">
-        <v>67</v>
-      </c>
-      <c r="F91" t="s">
-        <v>105</v>
-      </c>
-      <c r="G91" t="s">
-        <v>145</v>
+        <v>66</v>
       </c>
       <c r="H91" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I91" t="s">
-        <v>233</v>
-      </c>
-      <c r="J91" t="s">
-        <v>275</v>
+        <v>235</v>
       </c>
     </row>
     <row r="92" spans="1:10">
       <c r="A92" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B92" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C92" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D92" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E92" t="s">
         <v>68</v>
       </c>
       <c r="F92" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="G92" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="H92" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I92" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J92" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
     </row>
     <row r="93" spans="1:10">
       <c r="A93" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B93" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C93" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D93" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E93" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F93" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G93" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H93" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I93" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="J93" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="94" spans="1:10">
       <c r="A94" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B94" t="s">
         <v>35</v>
       </c>
       <c r="C94" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D94" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E94" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F94" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="G94" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="H94" t="s">
+        <v>150</v>
+      </c>
+      <c r="I94" t="s">
+        <v>238</v>
+      </c>
+      <c r="J94" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10">
+      <c r="A95" t="s">
+        <v>33</v>
+      </c>
+      <c r="B95" t="s">
+        <v>35</v>
+      </c>
+      <c r="C95" t="s">
+        <v>42</v>
+      </c>
+      <c r="D95" t="s">
+        <v>47</v>
+      </c>
+      <c r="E95" t="s">
+        <v>70</v>
+      </c>
+      <c r="F95" t="s">
+        <v>108</v>
+      </c>
+      <c r="G95" t="s">
         <v>148</v>
       </c>
-      <c r="I94" t="s">
-        <v>236</v>
-      </c>
-      <c r="J94" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10">
-      <c r="B95" t="s">
-        <v>36</v>
-      </c>
-      <c r="C95" t="s">
-        <v>40</v>
-      </c>
-      <c r="D95" t="s">
-        <v>45</v>
-      </c>
-      <c r="F95" t="s">
-        <v>70</v>
-      </c>
-      <c r="G95" t="s">
-        <v>109</v>
-      </c>
       <c r="H95" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I95" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J95" t="s">
-        <v>239</v>
+        <v>280</v>
       </c>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="B96" t="s">
+        <v>37</v>
+      </c>
+      <c r="C96" t="s">
+        <v>42</v>
+      </c>
+      <c r="D96" t="s">
+        <v>47</v>
       </c>
       <c r="E96" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F96" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G96" t="s">
-        <v>147</v>
+        <v>129</v>
+      </c>
+      <c r="H96" t="s">
+        <v>150</v>
       </c>
       <c r="I96" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J96" t="s">
-        <v>277</v>
+        <v>262</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10">
+      <c r="B97" t="s">
+        <v>38</v>
+      </c>
+      <c r="C97" t="s">
+        <v>42</v>
+      </c>
+      <c r="D97" t="s">
+        <v>47</v>
+      </c>
+      <c r="F97" t="s">
+        <v>72</v>
+      </c>
+      <c r="G97" t="s">
+        <v>111</v>
+      </c>
+      <c r="H97" t="s">
+        <v>150</v>
+      </c>
+      <c r="I97" t="s">
+        <v>241</v>
+      </c>
+      <c r="J97" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10">
+      <c r="A98" t="s">
+        <v>34</v>
+      </c>
+      <c r="E98" t="s">
+        <v>56</v>
+      </c>
+      <c r="F98" t="s">
+        <v>110</v>
+      </c>
+      <c r="G98" t="s">
+        <v>149</v>
+      </c>
+      <c r="I98" t="s">
+        <v>242</v>
+      </c>
+      <c r="J98" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update fix logika ekstraski tgl ro dan tgl muat
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -70,7 +70,7 @@
     <t>10 / 02 / 2026</t>
   </si>
   <si>
-    <t>02 . 00 / 10</t>
+    <t>02 : 00 100226</t>
   </si>
   <si>
     <t>11 februari 2026</t>
@@ -94,7 +94,7 @@
     <t>3 maret 2026</t>
   </si>
   <si>
-    <t>03 : 00 / 04</t>
+    <t>03 : 00 04032026</t>
   </si>
   <si>
     <t>03 maret 2026</t>
@@ -118,7 +118,7 @@
     <t>06 maret 2026</t>
   </si>
   <si>
-    <t>18 : 00 / 05</t>
+    <t>18 : 00 05022026</t>
   </si>
   <si>
     <t>2</t>
@@ -649,7 +649,7 @@
 NO HP :</t>
   </si>
   <si>
-    <t>Waktu loading :  02.00/10
+    <t>Waktu loading : 02:00 10-02-26
 Rute/tujuan : SRG-CGK
 Driver : Supriadi
 Nopol : B 9586 TXV
@@ -828,7 +828,7 @@
 No hp  : 085218843366</t>
   </si>
   <si>
-    <t>Waktu loading :  03:00/04
+    <t>Waktu loading : 03:00 04-03-2026
 Rute/tujuan : CGK - MES 
 driver  :
 Nopol  :
@@ -974,7 +974,7 @@
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading :  17:00/05
+    <t>Waktu loading : 17:00 05-03-2026
 Rute/tujuan : CGK - SUB
 driver  : Iwan Hariono
 Nopol  : BL 8188 JP
@@ -1067,7 +1067,7 @@
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading :  18:00/05
+    <t>Waktu loading : 18:00 05-02-2026
 Rute/tujuan : CGK - PKU
 driver  : Syarial
 Nopol  :BM 8486 AU

</xml_diff>

<commit_message>
fix bug record quantity for batch upload
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
   <si>
     <t>DATE</t>
   </si>
@@ -46,71 +46,156 @@
     <t>PHONE</t>
   </si>
   <si>
-    <t>06 maret 2026</t>
-  </si>
-  <si>
-    <t>18 : 00 05022026</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>04 mar 2026</t>
+  </si>
+  <si>
+    <t>05 mar 26</t>
+  </si>
+  <si>
+    <t>03 : 00 06 mar 26</t>
+  </si>
+  <si>
+    <t>05 maret 2026</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
+    <t>twb cbm</t>
+  </si>
+  <si>
+    <t>cddl</t>
+  </si>
+  <si>
     <t>twb</t>
   </si>
   <si>
+    <t>jne</t>
+  </si>
+  <si>
+    <t>cikokol</t>
+  </si>
+  <si>
     <t>argopantes</t>
   </si>
   <si>
-    <t>cgksub</t>
-  </si>
-  <si>
-    <t>cgk pku</t>
+    <t>suxcgk</t>
+  </si>
+  <si>
+    <t>cikarang</t>
+  </si>
+  <si>
+    <t>cgkpsr</t>
   </si>
   <si>
     <t>wahyudi</t>
   </si>
   <si>
-    <t>syarial</t>
+    <t>miyanta</t>
+  </si>
+  <si>
+    <t>davit</t>
+  </si>
+  <si>
+    <t>iwan hariono</t>
+  </si>
+  <si>
+    <t>akiyat</t>
   </si>
   <si>
     <t>n 9549 ua</t>
   </si>
   <si>
-    <t>bm 8486 au</t>
+    <t>f 9647 fh</t>
+  </si>
+  <si>
+    <t>b 9726 sxw</t>
+  </si>
+  <si>
+    <t>bl 8188 jp</t>
+  </si>
+  <si>
+    <t>l 9722 ue</t>
   </si>
   <si>
     <t>segera</t>
   </si>
   <si>
-    <t>REQUER ORDER ULANG DAN TAMBAHAN ON CALL
-06 MARET 2026
-3 UNIT TWB 50 CBM
- Lokasi : ARGOPANTES
-Rute / tujuan : CGK-SUB</t>
-  </si>
-  <si>
-    <t>Waktu loading : SEGERA
-Nama 	: Wahyudi
-Nopol		: N 9549 UA
-No Tlp	:085784422398
+    <t>Request Order Oncall  04 Mar 2026
+2 UNIT TWB 50 CBM
+Lokasi : JNE SURABAYA
+Rute/ Tujuan   : SUX-CGK</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 04 Mar 2026
+NAMA   : Wahyudi
+NOPOL : N 9549 UA
+NO HP : 085784422398
+Request Unit On Call Tgl 05 Mar 26
+1 Unit  Cddl / 24 Cbm
+Lokasi : Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : 06:00 06 Mar 26
+Rute/tujuan : CKR-JBR
+Driver   : miyanta
+Nopol  : F 9647 FH
+No Hp  :08118558105
+Request Unit On Call Tgl 05 Mar 26
+RAFAY
+1 Unit  Cddl / 24 Cbm
+Lokasi : Cikokol + Cikarang</t>
+  </si>
+  <si>
+    <t>Waktu loading : 03:00 06  Mar 26
+Rute/tujuan : CGK-PSR
+Driver   : Davit
+Nopol  : B 9726 SXW
+No Hp  :082117275166</t>
+  </si>
+  <si>
+    <t>REQUEST ORDER ONCALL
+05 MARET 2026:
 5 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES</t>
   </si>
   <si>
-    <t>Waktu loading : 18:00 05-02-2026
-Rute/tujuan : CGK - PKU
-driver  : Syarial
-Nopol  :BM 8486 AU
-No Hp :081317708658</t>
+    <t>Waktu loading : 17:00 05-03-2026
+Rute/tujuan : CGK - SUB
+driver  : Iwan Hariono
+Nopol  : BL 8188 JP
+No Hp :081389976421
+Request Order Oncall  05 Maret  2026
+2 UNIT TWB 50 CBM
+Lokasi : JNE SURABAYA
+Rute/ Tujuan   : SUX-CGK</t>
+  </si>
+  <si>
+    <t>Waktu loading : SEGERA 05 Maret  2026
+Driver : Akiyat
+Nopol : L 9722 UE
+No HP :081281122738</t>
   </si>
   <si>
     <t>085784422398</t>
   </si>
   <si>
-    <t>081317708658</t>
+    <t>08118558105</t>
+  </si>
+  <si>
+    <t>082117275166</t>
+  </si>
+  <si>
+    <t>081389976421</t>
+  </si>
+  <si>
+    <t>081281122738</t>
   </si>
 </sst>
 </file>
@@ -468,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -508,65 +593,160 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>11</v>
       </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>27</v>
+      <c r="D6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
+      </c>
+      <c r="J7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
undo db and batch logic, update filter and job number fitur, upgrade extraction acucation
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="117">
   <si>
     <t>DATE</t>
   </si>
@@ -46,25 +46,40 @@
     <t>PHONE</t>
   </si>
   <si>
-    <t>04 mar 2026</t>
-  </si>
-  <si>
-    <t>05 mar 26</t>
-  </si>
-  <si>
-    <t>03 : 00 06 mar 26</t>
-  </si>
-  <si>
-    <t>05 maret 2026</t>
+    <t>04 febuari 2026</t>
+  </si>
+  <si>
+    <t>05 / 02 / 2026</t>
+  </si>
+  <si>
+    <t>04 februari 2026</t>
+  </si>
+  <si>
+    <t>05 februari 2026</t>
+  </si>
+  <si>
+    <t>05 februari 2025</t>
+  </si>
+  <si>
+    <t>05 feb 26</t>
+  </si>
+  <si>
+    <t>06 febuary 2026</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>5</t>
+    <t>3</t>
   </si>
   <si>
     <t>twb cbm</t>
@@ -73,129 +88,484 @@
     <t>cddl</t>
   </si>
   <si>
+    <t>cbm</t>
+  </si>
+  <si>
     <t>twb</t>
   </si>
   <si>
-    <t>jne</t>
+    <t>argopantes</t>
+  </si>
+  <si>
+    <t>megahub</t>
   </si>
   <si>
     <t>cikokol</t>
   </si>
   <si>
-    <t>argopantes</t>
-  </si>
-  <si>
-    <t>suxcgk</t>
-  </si>
-  <si>
     <t>cikarang</t>
   </si>
   <si>
-    <t>cgkpsr</t>
+    <t>jne sub</t>
+  </si>
+  <si>
+    <t>cgk pdg</t>
+  </si>
+  <si>
+    <t>cgk jateng</t>
+  </si>
+  <si>
+    <t>cgk sub</t>
+  </si>
+  <si>
+    <t>cgk dps</t>
+  </si>
+  <si>
+    <t>cgk tkg</t>
+  </si>
+  <si>
+    <t>cgk plm</t>
+  </si>
+  <si>
+    <t>cgk pku</t>
+  </si>
+  <si>
+    <t>cgk mes</t>
+  </si>
+  <si>
+    <t>ckrjateng</t>
+  </si>
+  <si>
+    <t>subcgk</t>
+  </si>
+  <si>
+    <t>sutrisno</t>
+  </si>
+  <si>
+    <t>karyadi</t>
+  </si>
+  <si>
+    <t>m syaichoni</t>
+  </si>
+  <si>
+    <t>agus</t>
+  </si>
+  <si>
+    <t>jatmiyanta</t>
+  </si>
+  <si>
+    <t>siswanto</t>
+  </si>
+  <si>
+    <t>feri irawan</t>
+  </si>
+  <si>
+    <t>hadi</t>
+  </si>
+  <si>
+    <t>a . sukur</t>
+  </si>
+  <si>
+    <t>akiyat</t>
+  </si>
+  <si>
+    <t>ryan</t>
+  </si>
+  <si>
+    <t>hendra s . p</t>
+  </si>
+  <si>
+    <t>sandri</t>
+  </si>
+  <si>
+    <t>apar rahmat</t>
+  </si>
+  <si>
+    <t>m . ibnu</t>
   </si>
   <si>
     <t>wahyudi</t>
   </si>
   <si>
-    <t>miyanta</t>
-  </si>
-  <si>
-    <t>davit</t>
-  </si>
-  <si>
-    <t>iwan hariono</t>
-  </si>
-  <si>
-    <t>akiyat</t>
+    <t>sofyan</t>
+  </si>
+  <si>
+    <t>bm 8364 au</t>
+  </si>
+  <si>
+    <t>ad 8517 ba</t>
+  </si>
+  <si>
+    <t>n 8872 rk</t>
+  </si>
+  <si>
+    <t>d 9667 af</t>
+  </si>
+  <si>
+    <t>f 9647 fh</t>
+  </si>
+  <si>
+    <t>b 9120 wxr</t>
+  </si>
+  <si>
+    <t>bk 8516 vv</t>
+  </si>
+  <si>
+    <t>b 9446 mv</t>
+  </si>
+  <si>
+    <t>b 9477 keu</t>
+  </si>
+  <si>
+    <t>l 9722 ue</t>
+  </si>
+  <si>
+    <t>b 9084 veh</t>
+  </si>
+  <si>
+    <t>d 9044 ag</t>
+  </si>
+  <si>
+    <t>be 9636 bu</t>
+  </si>
+  <si>
+    <t>e9406hb</t>
+  </si>
+  <si>
+    <t>l 9511 al</t>
   </si>
   <si>
     <t>n 9549 ua</t>
   </si>
   <si>
-    <t>f 9647 fh</t>
-  </si>
-  <si>
-    <t>b 9726 sxw</t>
-  </si>
-  <si>
-    <t>bl 8188 jp</t>
-  </si>
-  <si>
-    <t>l 9722 ue</t>
+    <t>b 9679 wt</t>
   </si>
   <si>
     <t>segera</t>
   </si>
   <si>
-    <t>Request Order Oncall  04 Mar 2026
+    <t>07 : 00</t>
+  </si>
+  <si>
+    <t>00 : 00</t>
+  </si>
+  <si>
+    <t>06 : 00</t>
+  </si>
+  <si>
+    <t>03 : 00</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call 04 FEBUARI 2026
+RAFAY
+1 UNIT TWB 50 Cbm
+Lokasi : ARGOPANTES
+Waktu loading : SEGERA 04 FEBUARI 2026
+Rute/tujuan : CGK- PDG
+driver  : SUTRISNO
+Nopol  : BM 8364 AU
+No hp  :0853-5388-6066</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 04 FEBRUARI 2026:
+RAFAY
+3 unit Cddl 24 Cbm
+Lokasi : Megahub
+REQUEST ORDER KHUSUS 05/02/2026
+Waktu loading : 07:00
+Rute/tujuan : CGK - JATENG
+driver  : KARYADI
+Nopol  : AD 8517 BA
+No hp  :085865762797</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES 
+Waktu loading : SEGERA
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+Waktu loading : 18:00
+Rute/tujuan : CGK - SUB
+driver  : m syaichoni
+Nopol  : N 8872 Rk
+No hp  : +62 812-3189-5971
+Waktu loading : 21:00
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+Waktu loading : 00:00
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+REQUEST ORDER KHUSUS 05/02/2026
+Waktu loading : 03:00
+Rute/tujuan : CGK -SUB
+driver  : Lailan
+Nopol  : S 9272 UP
+No hp  : +62 878-8686-1780</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST TAMBAHAN ORDER ONCALL 04 FEBRUARI 2026:
+RAFAY
 2 UNIT TWB 50 CBM
-Lokasi : JNE SURABAYA
-Rute/ Tujuan   : SUX-CGK</t>
-  </si>
-  <si>
-    <t>Waktu loading : SEGERA 04 Mar 2026
-NAMA   : Wahyudi
-NOPOL : N 9549 UA
-NO HP : 085784422398
-Request Unit On Call Tgl 05 Mar 26
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 04 FEBRUARI 2026
+Rute/tujuan : CGK - SUB
+driver  : AGUS
+Nopol  : D 9667 AF
+No hp  :08817021866
+Rev plat nomor pak @Nomor tidak dikenal @Nomor tidak dikenal @Nomor tidak dikenal ðŸ™ðŸ»</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 04 FEBRUARI 2026:
+RAFAY
+1 unit Cddl 24 Cbm
+Lokasi : Megahub
+Waktu loading : SEGERA 04 FEBRUARI 2026
+Rute/tujuan : CGK - DPS
+driver 1 : Edi setiawan
+No hp  :0881023544597 
+Driver2 : Jatmiyanta
+No hp  :082118558105
+Nopol : F 9647 FH</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - TKG
+driver  :
+Nopol  :
+No hp  :</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - PLM
+driver  :
+Nopol  :
+No hp  :</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - PKU
+driver  : Siswanto
+Nopol  : B 9120 WXR
+No hp  : 081943564062
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - PKU
+driver  : 
+Nopol  : 
+No hp  :</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - MES
+driver  : feri irawan
+Nopol  : BK 8516 VV
+No hp  : 085219216210</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+RAFAY
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - MES
+driver  : HADI
+Nopol  :B 9446 MV
+No hp  :+62 831-9621-8655</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+RAFAY
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - MES
+driver  : A. Sukur 
+Nopol  :B 9477 KEU
+No hp  : 083169525183</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES 
+Waktu loading : SEGERA
+Rute/tujuan : CGK - SUB
+RAFAY
+driver  : AKIYAT
+Nopol  : L 9722 UE
+No hp  :081281122738</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2025
+RAFAY
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2025
+Rute/tujuan : CGK - PKU
+driver  : RYAN
+Nopol  : B 9084 VEH
+No hp  : 087837496810</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+5 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES 
+Waktu loading : SEGERA
+Rute/tujuan : CGK - SUB
+driver  : HENDRA S.P
+Nopol  : D 9044 AG
+No hp  : +62 877-8667-6177
+Waktu loading : 18:00
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+Waktu loading : 21:00
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+Waktu loading : 00:00
+Rute/tujuan : CGK - SUB
+driver  :
+Nopol  :
+No hp  :
+REQUEST ORDER KHUSUS 06/02/2026
+Waktu loading : 03:00
+Rute/tujuan : CGK -SUB
+driver  :
+Nopol  :
+No hp  :</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 05 FEBRUARI 2026:
+2 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 05 FEBRUARI 2026
+Rute/tujuan : CGK - PLM
+driver  : SANDRI
+Nopol  : BE 9636 BU
+No hp  :+62 889-0702-0037</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 05 Feb 26
+2 Unit  Cddl / 24 Cbm
+Lokasi : Cikarang
+Waktu loading : 06:00 06-02-26
+Rute/tujuan : CKR-Jateng Tentative
+Driver   : 
+Nopol  : 
+No Hp  :</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 05 Feb 26
 1 Unit  Cddl / 24 Cbm
-Lokasi : Cikarang</t>
-  </si>
-  <si>
-    <t>Waktu loading : 06:00 06 Mar 26
-Rute/tujuan : CKR-JBR
-Driver   : miyanta
-Nopol  : F 9647 FH
-No Hp  :08118558105
-Request Unit On Call Tgl 05 Mar 26
+Lokasi : Cikarang
+Waktu loading : 03:00 06-02-26
+Rute/tujuan : CKR-Jateng Tentative
+Nama : Apar Rahmat 
+Nopol : E9406HB 
+NO TLP : 085971812879</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 06 febuary 2026
 RAFAY
-1 Unit  Cddl / 24 Cbm
-Lokasi : Cikokol + Cikarang</t>
-  </si>
-  <si>
-    <t>Waktu loading : 03:00 06  Mar 26
-Rute/tujuan : CGK-PSR
-Driver   : Davit
-Nopol  : B 9726 SXW
-No Hp  :082117275166</t>
-  </si>
-  <si>
-    <t>REQUEST ORDER ONCALL
-05 MARET 2026:
-5 UNIT TWB 50 CBM
-Lokasi : ARGOPANTES</t>
-  </si>
-  <si>
-    <t>Waktu loading : 17:00 05-03-2026
-Rute/tujuan : CGK - SUB
-driver  : Iwan Hariono
-Nopol  : BL 8188 JP
-No Hp :081389976421
-Request Order Oncall  05 Maret  2026
-2 UNIT TWB 50 CBM
-Lokasi : JNE SURABAYA
-Rute/ Tujuan   : SUX-CGK</t>
-  </si>
-  <si>
-    <t>Waktu loading : SEGERA 05 Maret  2026
-Driver : Akiyat
-Nopol : L 9722 UE
-No HP :081281122738</t>
+3 unit twb 50 CBM
+Lokasi : ARGOPANTES 
+Waktu loading : SEGERA 06 febuary 2026
+Rute/tujuan : CGK- SUB
+driver  : M. iBNU
+Nopol  : L 9511 AL
+No hp  :082191633212</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 06 febuary 2026
+2 unit twb 50 CBM
+Lokasi : JNE SUB
+Waktu loading : SEGERA 06 febuary 2026
+Rute/tujuan : SUB-CGK
+driver  : WAHYUDI
+Nopol  : N 9549 UA
+No hp  :085784422398</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 06 febuary 2026
+2 unit twb 50 CBM
+Lokasi : JNE SUB
+Waktu loading : SEGERA 06 febuary 2026
+Rute/tujuan : SUB-CGK
+driver  : SOFYAN
+Nopol  : B 9679 WT
+No hp  : 082231837381</t>
+  </si>
+  <si>
+    <t>085353886066</t>
+  </si>
+  <si>
+    <t>085865762797</t>
+  </si>
+  <si>
+    <t>0 81231895971</t>
+  </si>
+  <si>
+    <t>08817021866</t>
+  </si>
+  <si>
+    <t>082118558105</t>
+  </si>
+  <si>
+    <t>081943564062</t>
+  </si>
+  <si>
+    <t>085219216210</t>
+  </si>
+  <si>
+    <t>0 83196218655</t>
+  </si>
+  <si>
+    <t>083169525183</t>
+  </si>
+  <si>
+    <t>081281122738</t>
+  </si>
+  <si>
+    <t>087837496810</t>
+  </si>
+  <si>
+    <t>0 87786676177</t>
+  </si>
+  <si>
+    <t>0 88907020037</t>
+  </si>
+  <si>
+    <t>085971812879</t>
+  </si>
+  <si>
+    <t>082191633212</t>
   </si>
   <si>
     <t>085784422398</t>
   </si>
   <si>
-    <t>08118558105</t>
-  </si>
-  <si>
-    <t>082117275166</t>
-  </si>
-  <si>
-    <t>081389976421</t>
-  </si>
-  <si>
-    <t>081281122738</t>
+    <t>082231837381</t>
   </si>
 </sst>
 </file>
@@ -553,7 +923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -593,19 +963,31 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" t="s">
+        <v>75</v>
       </c>
       <c r="I2" t="s">
-        <v>37</v>
+        <v>80</v>
+      </c>
+      <c r="J2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -613,94 +995,124 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
       </c>
       <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I3" t="s">
+        <v>81</v>
+      </c>
+      <c r="J3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
+      <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="G3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G4" t="s">
-        <v>32</v>
+        <v>60</v>
+      </c>
+      <c r="H4" t="s">
+        <v>77</v>
       </c>
       <c r="I4" t="s">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>12</v>
       </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="J5" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" t="s">
+        <v>75</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>84</v>
+      </c>
+      <c r="J6" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -708,45 +1120,446 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
+        <v>75</v>
       </c>
       <c r="I7" t="s">
-        <v>42</v>
-      </c>
-      <c r="J7" t="s">
-        <v>47</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="F8" t="s">
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" t="s">
+        <v>75</v>
+      </c>
+      <c r="I8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9" t="s">
+        <v>87</v>
+      </c>
+      <c r="J9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" t="s">
+        <v>89</v>
+      </c>
+      <c r="J11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13" t="s">
+        <v>91</v>
+      </c>
+      <c r="J13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" t="s">
+        <v>75</v>
+      </c>
+      <c r="I14" t="s">
+        <v>92</v>
+      </c>
+      <c r="J14" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" t="s">
+        <v>75</v>
+      </c>
+      <c r="I16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J16" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" t="s">
+        <v>78</v>
+      </c>
+      <c r="I17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" t="s">
+        <v>39</v>
+      </c>
+      <c r="F18" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" t="s">
+        <v>71</v>
+      </c>
+      <c r="H18" t="s">
+        <v>79</v>
+      </c>
+      <c r="I18" t="s">
+        <v>96</v>
+      </c>
+      <c r="J18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="s">
+        <v>75</v>
+      </c>
+      <c r="I19" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
         <v>30</v>
       </c>
-      <c r="G8" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" t="s">
-        <v>36</v>
-      </c>
-      <c r="I8" t="s">
-        <v>43</v>
-      </c>
-      <c r="J8" t="s">
-        <v>48</v>
+      <c r="E20" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" t="s">
+        <v>56</v>
+      </c>
+      <c r="G20" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20" t="s">
+        <v>75</v>
+      </c>
+      <c r="I20" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" t="s">
+        <v>75</v>
+      </c>
+      <c r="I21" t="s">
+        <v>99</v>
+      </c>
+      <c r="J21" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
integrate db with incremental logic
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="120">
   <si>
     <t>DATE</t>
   </si>
@@ -52,15 +52,24 @@
     <t>05 / 02 / 2026</t>
   </si>
   <si>
+    <t>09 maret 2026</t>
+  </si>
+  <si>
     <t>04 februari 2026</t>
   </si>
   <si>
     <t>05 februari 2026</t>
   </si>
   <si>
+    <t>7 / 3 / 2026</t>
+  </si>
+  <si>
     <t>05 februari 2025</t>
   </si>
   <si>
+    <t>7 / 02 / 2026</t>
+  </si>
+  <si>
     <t>05 feb 26</t>
   </si>
   <si>
@@ -88,12 +97,12 @@
     <t>cddl</t>
   </si>
   <si>
+    <t>twb</t>
+  </si>
+  <si>
     <t>cbm</t>
   </si>
   <si>
-    <t>twb</t>
-  </si>
-  <si>
     <t>argopantes</t>
   </si>
   <si>
@@ -247,7 +256,7 @@
     <t>07 : 00</t>
   </si>
   <si>
-    <t>00 : 00</t>
+    <t>21</t>
   </si>
   <si>
     <t>06 : 00</t>
@@ -279,25 +288,25 @@
 No hp  :085865762797</t>
   </si>
   <si>
-    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
+    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL 09 MARET 2026
 5 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES 
-Waktu loading : SEGERA
+Waktu loading : SEGERA 09 MARET 2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
 No hp  :
-Waktu loading : 18:00
+Waktu loading : 18:00 09 MARET 2026
 Rute/tujuan : CGK - SUB
 driver  : m syaichoni
 Nopol  : N 8872 Rk
 No hp  : +62 812-3189-5971
-Waktu loading : 21:00
+Waktu loading : 21:00 09 MARET 2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
 No hp  :
-Waktu loading : 00:00
+Waktu loading : 00:00 09 MARET 2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
@@ -318,8 +327,7 @@
 Rute/tujuan : CGK - SUB
 driver  : AGUS
 Nopol  : D 9667 AF
-No hp  :08817021866
-Rev plat nomor pak @Nomor tidak dikenal @Nomor tidak dikenal @Nomor tidak dikenal ðŸ™ðŸ»</t>
+No hp  :08817021866</t>
   </si>
   <si>
     <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 04 FEBRUARI 2026:
@@ -406,7 +414,7 @@
     <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
 5 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES 
-Waktu loading : SEGERA
+Waktu loading : SEGERA 7/3/2026
 Rute/tujuan : CGK - SUB
 RAFAY
 driver  : AKIYAT
@@ -428,22 +436,22 @@
     <t>[WA_TS] Akbar Rafay: REQUEST ORDER ULANG ONCALL
 5 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES 
-Waktu loading : SEGERA
+Waktu loading : SEGERA 7/02/2026
 Rute/tujuan : CGK - SUB
 driver  : HENDRA S.P
 Nopol  : D 9044 AG
 No hp  : +62 877-8667-6177
-Waktu loading : 18:00
+Waktu loading : 18:00 7/02/2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
 No hp  :
-Waktu loading : 21:00
+Waktu loading : 21:00 7/02/2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
 No hp  :
-Waktu loading : 00:00
+Waktu loading : 00:00 7/02/2026
 Rute/tujuan : CGK - SUB
 driver  :
 Nopol  :
@@ -963,31 +971,31 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -995,571 +1003,580 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="J5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="J6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I7" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H8" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J9" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="J10" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" t="s">
+        <v>93</v>
+      </c>
+      <c r="J12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
         <v>28</v>
       </c>
-      <c r="E12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" t="s">
-        <v>66</v>
-      </c>
-      <c r="H12" t="s">
-        <v>75</v>
-      </c>
-      <c r="I12" t="s">
-        <v>90</v>
-      </c>
-      <c r="J12" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>24</v>
-      </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" t="s">
+        <v>95</v>
+      </c>
+      <c r="J14" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
         <v>22</v>
       </c>
-      <c r="D14" t="s">
+      <c r="C15" t="s">
         <v>28</v>
       </c>
-      <c r="E14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" t="s">
-        <v>51</v>
-      </c>
-      <c r="G14" t="s">
-        <v>68</v>
-      </c>
-      <c r="H14" t="s">
-        <v>75</v>
-      </c>
-      <c r="I14" t="s">
-        <v>92</v>
-      </c>
-      <c r="J14" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
       <c r="D15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="I15" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J15" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F16" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="J16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E17" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H17" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D18" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H18" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I18" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J18" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F19" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H19" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I19" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="J19" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F20" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I20" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="J20" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G21" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I21" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="J21" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix typo normalization feature and tuning tgl ro dan tgl muat for variation tgl muat in one order
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>DATE</t>
   </si>
@@ -46,180 +46,54 @@
     <t>PHONE</t>
   </si>
   <si>
-    <t>3 maret 2026</t>
-  </si>
-  <si>
-    <t>03 maret 2026</t>
-  </si>
-  <si>
-    <t>04 maret 2026</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>cbm</t>
-  </si>
-  <si>
-    <t>cddl</t>
-  </si>
-  <si>
-    <t>twb 50 cbm</t>
+    <t>05 / 02</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>twb cbm</t>
   </si>
   <si>
     <t>argopantes</t>
   </si>
   <si>
-    <t>megahub</t>
-  </si>
-  <si>
-    <t>argo pantes</t>
-  </si>
-  <si>
-    <t>sub cgk</t>
-  </si>
-  <si>
-    <t>cgk jatim</t>
-  </si>
-  <si>
-    <t>cgk jateng tentatif</t>
-  </si>
-  <si>
-    <t>cgk pku</t>
-  </si>
-  <si>
-    <t>cgk mes</t>
-  </si>
-  <si>
-    <t>yuda</t>
-  </si>
-  <si>
-    <t>ari purnama</t>
-  </si>
-  <si>
-    <t>dedeng</t>
-  </si>
-  <si>
-    <t>jupri</t>
-  </si>
-  <si>
-    <t>misno</t>
-  </si>
-  <si>
-    <t>usman afandi</t>
-  </si>
-  <si>
-    <t>w 8973 uq</t>
-  </si>
-  <si>
-    <t>b 9383 txv</t>
-  </si>
-  <si>
-    <t>e 9426 aa</t>
-  </si>
-  <si>
-    <t>bm 9273 ro</t>
-  </si>
-  <si>
-    <t>bn 8038 rp</t>
-  </si>
-  <si>
-    <t>be 8456 fn</t>
+    <t>cgk pdg</t>
+  </si>
+  <si>
+    <t>ahmad</t>
+  </si>
+  <si>
+    <t>bm 8364 bb</t>
   </si>
   <si>
     <t>segera</t>
   </si>
   <si>
-    <t>REQUEST  ORDER  ONCALL  3 MARET 2026
-1 UNIT WB/50 CBM
-Lokasi : ARGOPANTES 
-Waktu loading : 23:00 3 MARET 2026
-Rute/tujuan : SUB - CGK
-driver  : Yuda
-Nopol  : W 8973 UQ
-No hp  : 089507296985</t>
-  </si>
-  <si>
-    <t>REQUEST ORDER ONCALL 03 maret 2026:
-3 unit Cddl 24 Cbm
-Lokasi : Megahub
-Waktu loading : 23:00 03 maret 2026
-Rute/tujuan : CGK - JATIM
-driver  : Ari purnama
-Nopol  : B 9383 TXV
-No hp : 082136689169
-Fyi pak  @Nomor tidak dikenal@Nomor tidak dikenal</t>
-  </si>
-  <si>
-    <t>REQUEST ULANG ORDER ONCALL 04 MARET 2026:
-8 unit Cddl 24 Cbm
-Lokasi : *argo pantes *
-Waktu loading : SEGERA 04 MARET 2026
-Rute/tujuan : *CGK - Jateng tentatif
-Nama : Dedeng
-Nopol :E 9426 Aa
-No.hp : 0895393659401</t>
-  </si>
-  <si>
-    <t>Request Unit On Call Tgl 04 Maret 2026
-5 UNIT TWB 50 CBM
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call 04 FEBUARI 2026
+RAFAY
+3 UNIT TWB 50 Cbm
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA 04 Maret 2026
-Rute/tujuan : CGK - PKU
-driver  : Jupri
-Nopol  : BM 9273 RO
-No Hp :082172471454</t>
-  </si>
-  <si>
-    <t>REQUEST ORDER ONCALL
-04 MARET 2026:
-5 UNIT TWB 50 CBM
+Waktu loading : SEGERA 04 FEBUARI 2026
+Rute/tujuan : CGK- PDG
+driver  : SUTRISNO
+Nopol  : BM 8364 AU
+No hp  :0853-5388-6066
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA
-Rute/tujuan : CGK - MES
-driver  : Andi
-Nopol  : BE 8610 DB
-No Hp :081374328877
-Waktu loading : SEGERA
-Rute/tujuan : CGK - MES
-driver  : Misno
-Nopol  : BN 8038 RP
-No Hp :082211762649</t>
-  </si>
-  <si>
-    <t>REQUEST ORDER ONCALL
-04 MARET 2026:
-5 UNIT TWB 50 CBM
+Waktu loading : SEGERA 04 FEBUARI 2026
+Rute/tujuan : CGK- PDG
+driver  : AHMAD
+Nopol  : BM 8364 BB
+No hp  :0853-5388-6077
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA
-Rute/tujuan : CGK - MES
-driver  : Usman Afandi
-Nopol  : BE 8456 FN
-No Hp : +62 853-7337-2594</t>
-  </si>
-  <si>
-    <t>089507296985</t>
-  </si>
-  <si>
-    <t>082136689169</t>
-  </si>
-  <si>
-    <t>0895393659401</t>
-  </si>
-  <si>
-    <t>082172471454</t>
-  </si>
-  <si>
-    <t>082211762649</t>
-  </si>
-  <si>
-    <t>0 85373372594</t>
+Waktu loading : 05/02/2026
+Rute/tujuan : CGK- PDG
+driver  : wahyudi
+Nopol  : BM 8364 BB
+No hp  :0853-5388-6077</t>
+  </si>
+  <si>
+    <t>085353886077</t>
   </si>
 </sst>
 </file>
@@ -577,7 +451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -617,185 +491,31 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
         <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" t="s">
-        <v>37</v>
-      </c>
-      <c r="H6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" t="s">
-        <v>44</v>
-      </c>
-      <c r="J6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update model machine learning untuk revisi dan refill logic
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>UNIT_QTY</t>
   </si>
@@ -49,9 +49,6 @@
     <t>RO_DATE</t>
   </si>
   <si>
-    <t>LOAD_DATE</t>
-  </si>
-  <si>
     <t>PHONE</t>
   </si>
   <si>
@@ -67,10 +64,10 @@
     <t>cgk sub</t>
   </si>
   <si>
-    <t>bagus</t>
-  </si>
-  <si>
-    <t>b 9563 taa</t>
+    <t>agung</t>
+  </si>
+  <si>
+    <t>bm 8364 uu</t>
   </si>
   <si>
     <t>segera</t>
@@ -79,35 +76,33 @@
     <t>NEW_ORDER</t>
   </si>
   <si>
-    <t>[WA_TS] Akbar Rafay: REQUEST ORDER ONCALL 12 FEBRUARI 2026:
-3 UNIT TWB 50 Cbm
+    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 12 MARET 2026
+RAFAY
+3 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA 12 FEBRUARI 2026
+Waktu loading : SEGERA 12 MARET 2026
 Rute/tujuan : CGK - SUB
-driver  : Rosyit
-Nopol  : B 9563 TEU
-No hp  : 082313572678
+driver  : ADE
+Nopol  : BM 8364 AA
+No hp  : 085353886066
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA 12 FEBRUARI 2026
+Waktu loading : SEGERA 12 MARET 2026
 Rute/tujuan : CGK - SUB
-driver  : BAGUS
-Nopol  : B 9563 TAA
-No hp  : 0823135882147
+driver  : AGUNG
+Nopol  : BM 8364 UU
+No hp  : 085353886066
 Lokasi : ARGOPANTES
-Waktu loading : SEGERA 12 FEBRUARI 2026
+Waktu loading : SEGERA 12 MARET 2026
 Rute/tujuan : CGK - SUB
-driver  : AJENG
-Nopol  : B 9563 TBB
-No hp  : 0823135882147</t>
-  </si>
-  <si>
-    <t>12 februari</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>0823135882147</t>
+driver  : ADRI
+Nopol  : BM 8364 BB
+No hp  : 085353886066</t>
+  </si>
+  <si>
+    <t>12 maret 2026</t>
+  </si>
+  <si>
+    <t>085353886066</t>
   </si>
 </sst>
 </file>
@@ -465,10 +460,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,49 +500,43 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2">
+        <v>0.9994</v>
+      </c>
+      <c r="J2" t="s">
         <v>20</v>
       </c>
-      <c r="I2">
-        <v>0.9995000000000001</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>22</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update switch revisi dan refill dominan ml
</commit_message>
<xml_diff>
--- a/output_orderan.xlsx
+++ b/output_orderan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="122">
   <si>
     <t>UNIT_QTY</t>
   </si>
@@ -49,60 +49,501 @@
     <t>RO_DATE</t>
   </si>
   <si>
+    <t>LOAD_DATE</t>
+  </si>
+  <si>
     <t>PHONE</t>
   </si>
   <si>
-    <t>3</t>
+    <t>1</t>
   </si>
   <si>
     <t>twb</t>
   </si>
   <si>
+    <t>cddl</t>
+  </si>
+  <si>
     <t>argopantes</t>
   </si>
   <si>
+    <t>cikokol</t>
+  </si>
+  <si>
+    <t>megahub</t>
+  </si>
+  <si>
+    <t>jne sub</t>
+  </si>
+  <si>
+    <t>cikarang</t>
+  </si>
+  <si>
     <t>cgk sub</t>
   </si>
   <si>
-    <t>agung</t>
-  </si>
-  <si>
-    <t>bm 8364 uu</t>
+    <t>cgk pku</t>
+  </si>
+  <si>
+    <t>cgk jateng</t>
+  </si>
+  <si>
+    <t>sub cgk</t>
+  </si>
+  <si>
+    <t>ckr jatim tentative</t>
+  </si>
+  <si>
+    <t>cgk dps</t>
+  </si>
+  <si>
+    <t>cgk plm</t>
+  </si>
+  <si>
+    <t>cgk mes</t>
+  </si>
+  <si>
+    <t>cgk bdg</t>
+  </si>
+  <si>
+    <t>cgk jepara</t>
+  </si>
+  <si>
+    <t>roni</t>
+  </si>
+  <si>
+    <t>dedi</t>
+  </si>
+  <si>
+    <t>sandri</t>
+  </si>
+  <si>
+    <t>hadi</t>
+  </si>
+  <si>
+    <t>apar rahmat</t>
+  </si>
+  <si>
+    <t>edi setiawan</t>
+  </si>
+  <si>
+    <t>sofyan</t>
+  </si>
+  <si>
+    <t>bayu</t>
+  </si>
+  <si>
+    <t>ryan</t>
+  </si>
+  <si>
+    <t>agus</t>
+  </si>
+  <si>
+    <t>lailan</t>
+  </si>
+  <si>
+    <t>akiyat</t>
+  </si>
+  <si>
+    <t>a sukur</t>
+  </si>
+  <si>
+    <t>mujito</t>
+  </si>
+  <si>
+    <t>usman afandi</t>
+  </si>
+  <si>
+    <t>yusni gunawan</t>
+  </si>
+  <si>
+    <t>samsul</t>
+  </si>
+  <si>
+    <t>rajiev fikri</t>
+  </si>
+  <si>
+    <t>dian saputra</t>
+  </si>
+  <si>
+    <t>supriyanto</t>
+  </si>
+  <si>
+    <t>b 9001 aa</t>
+  </si>
+  <si>
+    <t>b 9002 ab</t>
+  </si>
+  <si>
+    <t>be 9636 bu</t>
+  </si>
+  <si>
+    <t>b 9446 mv</t>
+  </si>
+  <si>
+    <t>e 9406 hb</t>
+  </si>
+  <si>
+    <t>f 9647 fh</t>
+  </si>
+  <si>
+    <t>b 9679 wt</t>
+  </si>
+  <si>
+    <t>l 9511 al</t>
+  </si>
+  <si>
+    <t>b 9084 veh</t>
+  </si>
+  <si>
+    <t>d 9667 af</t>
+  </si>
+  <si>
+    <t>s 9272 up</t>
+  </si>
+  <si>
+    <t>l 9722 ue</t>
+  </si>
+  <si>
+    <t>b 9477 keu</t>
+  </si>
+  <si>
+    <t>be 8837 gk</t>
+  </si>
+  <si>
+    <t>be 8456 fn</t>
+  </si>
+  <si>
+    <t>be 8951 by</t>
+  </si>
+  <si>
+    <t>b 9771 uew</t>
+  </si>
+  <si>
+    <t>b 9591 uxx</t>
+  </si>
+  <si>
+    <t>be 8334 gba</t>
+  </si>
+  <si>
+    <t>be 8940 db</t>
   </si>
   <si>
     <t>segera</t>
   </si>
   <si>
+    <t>07 : 00</t>
+  </si>
+  <si>
+    <t>06 : 00</t>
+  </si>
+  <si>
+    <t>21 : 00</t>
+  </si>
+  <si>
+    <t>18 : 00</t>
+  </si>
+  <si>
+    <t>00 : 00</t>
+  </si>
+  <si>
     <t>NEW_ORDER</t>
   </si>
   <si>
-    <t>[WA_TS] Akbar Rafay: Request Unit On Call Tgl 12 MARET 2026
-RAFAY
-3 UNIT TWB 50 CBM
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES
 Waktu loading : SEGERA 12 MARET 2026
 Rute/tujuan : CGK - SUB
-driver  : ADE
-Nopol  : BM 8364 AA
-No hp  : 085353886066
+driver  : RONI
+Nopol  : B 9001 AA
+No hp  : 081311110001</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES
 Waktu loading : SEGERA 12 MARET 2026
 Rute/tujuan : CGK - SUB
-driver  : AGUNG
-Nopol  : BM 8364 UU
-No hp  : 085353886066
+driver  : DEDI
+Nopol  : B 9002 AB
+No hp  : 081311110002</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : CGK - PKU
+driver  : SANDRI
+Nopol  : BE 9636 BU
+No hp  : 088907020037</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : CGK - PKU
+driver  : HADI
+Nopol  : B 9446 MV
+No hp  : 083196218655</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : MEGAHUB
+REQUEST ORDER KHUSUS 13/03/2026
+Waktu loading : 07:00
+Rute/tujuan : CGK - JATENG
+driver  : APAR RAHMAT
+Nopol  : E 9406 HB
+No hp  : 085971812879</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : MEGAHUB
+REQUEST ORDER KHUSUS 13/03/2026
+Waktu loading : 07:00
+Rute/tujuan : CGK - JATENG
+driver  : EDI SETIAWAN
+Nopol  : F 9647 FH
+No hp  : 0881023544597</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : JNE SUB
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : SUB - CGK
+driver  : SOFYAN
+Nopol  : B 9679 WT
+No hp  : 082231837381</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : JNE SUB
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : SUB - CGK
+driver  : BAYU
+Nopol  : L 9511 AL
+No hp  : 082191633212</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : CIKARANG
+Waktu loading : 06:00 13-03-26
+Rute/tujuan : CKR - JATIM TENTATIVE
+driver  : RYAN
+Nopol  : B 9084 VEH
+No hp  : 087837496810</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : CIKARANG
+Waktu loading : 06:00 13-03-26
+Rute/tujuan : CKR - JATIM TENTATIVE
+driver  : AGUS
+Nopol  : D 9667 AF
+No hp  : 08817021866</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
 Lokasi : ARGOPANTES
+Waktu loading : 21:00 12 MARET 2026
+Rute/tujuan : CGK - DPS
+driver  : LAILAN
+Nopol  : S 9272 UP
+No hp  : 087886861780</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES
+Waktu loading : 21:00 12 MARET 2026
+Rute/tujuan : CGK - DPS
+driver  : AKIYAT
+Nopol  : L 9722 UE
+No hp  : 081281122738</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
 Waktu loading : SEGERA 12 MARET 2026
-Rute/tujuan : CGK - SUB
-driver  : ADRI
-Nopol  : BM 8364 BB
-No hp  : 085353886066</t>
+Rute/tujuan : CGK - PLM
+driver  : A SUKUR
+Nopol  : B 9477 KEU
+No hp  : 083169525183</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : CGK - PLM
+driver  : MUJITO
+Nopol  : BE 8837 GK
+No hp  : 082275004149</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : CGK - MES
+driver  : USMAN AFANDI
+Nopol  : BE 8456 FN
+No hp  : 082382200400</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : CIKOKOL
+Waktu loading : SEGERA 12 MARET 2026
+Rute/tujuan : CGK - MES
+driver  : YUSNI GUNAWAN
+Nopol  : BE 8951 BY
+No hp  : 085729113217</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : MEGAHUB
+Waktu loading : 18:00 12 MARET 2026
+Rute/tujuan : CGK - BDG
+driver  : SAMSUL
+Nopol  : B 9771 UEW
+No hp  : 082234567802</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT CDDL 24 CBM
+Lokasi : MEGAHUB
+Waktu loading : 18:00 12 MARET 2026
+Rute/tujuan : CGK - BDG
+driver  : RAJIEV FIKRI
+Nopol  : B 9591 UXX
+No hp  : 082234567803</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES
+REQUEST ORDER KHUSUS 13/03/2026
+Waktu loading : 00:00
+Rute/tujuan : CGK - JEPARA
+driver  : DIAN SAPUTRA
+Nopol  : BE 8334 GBA
+No hp  : 081262189242</t>
+  </si>
+  <si>
+    <t>[WA_TS] Akbar Rafay: REQUEST ULANG ORDER ONCALL 12 MARET 2026
+RAFAY
+1 UNIT TWB 50 CBM
+Lokasi : ARGOPANTES
+REQUEST ORDER KHUSUS 13/03/2026
+Waktu loading : 00:00
+Rute/tujuan : CGK - JEPARA
+driver  : SUPRIYANTO
+Nopol  : BE 8940 DB
+No hp  : 082164544736</t>
   </si>
   <si>
     <t>12 maret 2026</t>
   </si>
   <si>
-    <t>085353886066</t>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13 / 03 / 2026</t>
+  </si>
+  <si>
+    <t>12 2026</t>
+  </si>
+  <si>
+    <t>081311110001</t>
+  </si>
+  <si>
+    <t>081311110002</t>
+  </si>
+  <si>
+    <t>088907020037</t>
+  </si>
+  <si>
+    <t>083196218655</t>
+  </si>
+  <si>
+    <t>085971812879</t>
+  </si>
+  <si>
+    <t>0881023544597</t>
+  </si>
+  <si>
+    <t>082231837381</t>
+  </si>
+  <si>
+    <t>082191633212</t>
+  </si>
+  <si>
+    <t>087837496810</t>
+  </si>
+  <si>
+    <t>08817021866</t>
+  </si>
+  <si>
+    <t>087886861780</t>
+  </si>
+  <si>
+    <t>081281122738</t>
+  </si>
+  <si>
+    <t>083169525183</t>
+  </si>
+  <si>
+    <t>082275004149</t>
+  </si>
+  <si>
+    <t>082382200400</t>
+  </si>
+  <si>
+    <t>085729113217</t>
+  </si>
+  <si>
+    <t>082234567802</t>
+  </si>
+  <si>
+    <t>082234567803</t>
+  </si>
+  <si>
+    <t>081262189242</t>
+  </si>
+  <si>
+    <t>082164544736</t>
   </si>
 </sst>
 </file>
@@ -460,10 +901,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -500,43 +941,822 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>77</v>
       </c>
       <c r="I2">
         <v>0.9994</v>
       </c>
       <c r="J2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" t="s">
+        <v>98</v>
+      </c>
+      <c r="M2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3">
+        <v>0.9994</v>
+      </c>
+      <c r="J3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" t="s">
+        <v>98</v>
+      </c>
+      <c r="L3" t="s">
+        <v>98</v>
+      </c>
+      <c r="M3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I4">
+        <v>0.9994</v>
+      </c>
+      <c r="J4" t="s">
+        <v>80</v>
+      </c>
+      <c r="K4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L4" t="s">
+        <v>99</v>
+      </c>
+      <c r="M4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" t="s">
+        <v>77</v>
+      </c>
+      <c r="I5">
+        <v>0.9993</v>
+      </c>
+      <c r="J5" t="s">
+        <v>81</v>
+      </c>
+      <c r="K5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L5" t="s">
+        <v>99</v>
+      </c>
+      <c r="M5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I6">
+        <v>0.9994</v>
+      </c>
+      <c r="J6" t="s">
+        <v>82</v>
+      </c>
+      <c r="K6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L6" t="s">
+        <v>100</v>
+      </c>
+      <c r="M6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I7">
+        <v>0.9994</v>
+      </c>
+      <c r="J7" t="s">
+        <v>83</v>
+      </c>
+      <c r="K7" t="s">
+        <v>98</v>
+      </c>
+      <c r="L7" t="s">
+        <v>100</v>
+      </c>
+      <c r="M7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" t="s">
+        <v>77</v>
+      </c>
+      <c r="I8">
+        <v>0.9994</v>
+      </c>
+      <c r="J8" t="s">
+        <v>84</v>
+      </c>
+      <c r="K8" t="s">
+        <v>98</v>
+      </c>
+      <c r="L8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" t="s">
+        <v>77</v>
+      </c>
+      <c r="I9">
+        <v>0.9994</v>
+      </c>
+      <c r="J9" t="s">
+        <v>85</v>
+      </c>
+      <c r="K9" t="s">
+        <v>98</v>
+      </c>
+      <c r="L9" t="s">
+        <v>99</v>
+      </c>
+      <c r="M9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
         <v>20</v>
       </c>
-      <c r="K2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" t="s">
-        <v>22</v>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10">
+        <v>0.9994</v>
+      </c>
+      <c r="J10" t="s">
+        <v>86</v>
+      </c>
+      <c r="K10" t="s">
+        <v>98</v>
+      </c>
+      <c r="M10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I11">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="J11" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" t="s">
+        <v>98</v>
+      </c>
+      <c r="M11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I12">
+        <v>0.9994</v>
+      </c>
+      <c r="J12" t="s">
+        <v>88</v>
+      </c>
+      <c r="K12" t="s">
+        <v>98</v>
+      </c>
+      <c r="L12" t="s">
+        <v>98</v>
+      </c>
+      <c r="M12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I13">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="J13" t="s">
+        <v>89</v>
+      </c>
+      <c r="K13" t="s">
+        <v>98</v>
+      </c>
+      <c r="L13" t="s">
+        <v>98</v>
+      </c>
+      <c r="M13" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14">
+        <v>0.9994</v>
+      </c>
+      <c r="J14" t="s">
+        <v>90</v>
+      </c>
+      <c r="K14" t="s">
+        <v>98</v>
+      </c>
+      <c r="L14" t="s">
+        <v>99</v>
+      </c>
+      <c r="M14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" t="s">
+        <v>71</v>
+      </c>
+      <c r="H15" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15">
+        <v>0.9994</v>
+      </c>
+      <c r="J15" t="s">
+        <v>91</v>
+      </c>
+      <c r="K15" t="s">
+        <v>98</v>
+      </c>
+      <c r="L15" t="s">
+        <v>99</v>
+      </c>
+      <c r="M15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" t="s">
+        <v>77</v>
+      </c>
+      <c r="I16">
+        <v>0.9993</v>
+      </c>
+      <c r="J16" t="s">
+        <v>92</v>
+      </c>
+      <c r="K16" t="s">
+        <v>98</v>
+      </c>
+      <c r="L16" t="s">
+        <v>101</v>
+      </c>
+      <c r="M16" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" t="s">
+        <v>66</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" t="s">
+        <v>77</v>
+      </c>
+      <c r="I17">
+        <v>0.9994</v>
+      </c>
+      <c r="J17" t="s">
+        <v>93</v>
+      </c>
+      <c r="K17" t="s">
+        <v>98</v>
+      </c>
+      <c r="L17" t="s">
+        <v>99</v>
+      </c>
+      <c r="M17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H18" t="s">
+        <v>77</v>
+      </c>
+      <c r="I18">
+        <v>0.9994</v>
+      </c>
+      <c r="J18" t="s">
+        <v>94</v>
+      </c>
+      <c r="K18" t="s">
+        <v>98</v>
+      </c>
+      <c r="L18" t="s">
+        <v>98</v>
+      </c>
+      <c r="M18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" t="s">
+        <v>68</v>
+      </c>
+      <c r="G19" t="s">
+        <v>75</v>
+      </c>
+      <c r="H19" t="s">
+        <v>77</v>
+      </c>
+      <c r="I19">
+        <v>0.9994</v>
+      </c>
+      <c r="J19" t="s">
+        <v>95</v>
+      </c>
+      <c r="K19" t="s">
+        <v>98</v>
+      </c>
+      <c r="L19" t="s">
+        <v>98</v>
+      </c>
+      <c r="M19" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" t="s">
+        <v>69</v>
+      </c>
+      <c r="G20" t="s">
+        <v>76</v>
+      </c>
+      <c r="H20" t="s">
+        <v>77</v>
+      </c>
+      <c r="I20">
+        <v>0.9994</v>
+      </c>
+      <c r="J20" t="s">
+        <v>96</v>
+      </c>
+      <c r="K20" t="s">
+        <v>98</v>
+      </c>
+      <c r="L20" t="s">
+        <v>100</v>
+      </c>
+      <c r="M20" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" t="s">
+        <v>76</v>
+      </c>
+      <c r="H21" t="s">
+        <v>77</v>
+      </c>
+      <c r="I21">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="J21" t="s">
+        <v>97</v>
+      </c>
+      <c r="K21" t="s">
+        <v>98</v>
+      </c>
+      <c r="L21" t="s">
+        <v>100</v>
+      </c>
+      <c r="M21" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>